<commit_message>
docs: mark WP4 done on the WBS.
Tasks 6.0-6.4 and the four backend-map acceptance rows now match PR #55.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/commercialization/Open-Notebook-Commercialization-WBS-Task-Schedule.xlsx
+++ b/docs/commercialization/Open-Notebook-Commercialization-WBS-Task-Schedule.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimating Assumptions" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'WBS Task List'!$A$5:$S$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'WBS Task List'!$A$5:$S$102</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -59,7 +59,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -94,11 +94,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E0E7FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
     <fill>
@@ -138,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -151,7 +146,7 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -192,13 +187,10 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -760,13 +752,13 @@
         <v>32</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>4</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.3125</v>
+        <v>0.375</v>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
@@ -871,7 +863,7 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>56</v>
+        <v>96</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
@@ -879,7 +871,7 @@
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>0</v>
@@ -931,16 +923,14 @@
       <c r="C14" s="3" t="n">
         <v>49</v>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D14" s="3" t="n">
+        <v>49</v>
       </c>
       <c r="E14" s="3" t="n">
         <v>6.2</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
@@ -1079,13 +1069,13 @@
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>1035</v>
+        <v>1075</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>439</v>
+        <v>489</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>0.4229951690821256</v>
+        <v>0.4546976744186046</v>
       </c>
     </row>
     <row r="22">
@@ -1102,7 +1092,7 @@
         </is>
       </c>
       <c r="B23" s="11" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="24">
@@ -1112,7 +1102,7 @@
         </is>
       </c>
       <c r="B24" s="11" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25">
@@ -1132,7 +1122,7 @@
         </is>
       </c>
       <c r="B26" s="11" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27">
@@ -1142,7 +1132,7 @@
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1152,7 +1142,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>597.2</v>
+        <v>586.2</v>
       </c>
     </row>
     <row r="29">
@@ -1162,7 +1152,7 @@
         </is>
       </c>
       <c r="B29" s="11" t="n">
-        <v>74.90000000000001</v>
+        <v>73.40000000000001</v>
       </c>
     </row>
     <row r="30">
@@ -1232,7 +1222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S101"/>
+  <dimension ref="A1:S102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4126,12 +4116,12 @@
           <t>Cleaner image; allowlist reduced</t>
         </is>
       </c>
-      <c r="F39" s="23" t="inlineStr">
-        <is>
-          <t>Blocked</t>
-        </is>
-      </c>
-      <c r="G39" s="24" t="inlineStr">
+      <c r="F39" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G39" s="23" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -4147,18 +4137,26 @@
       <c r="J39" s="17" t="n">
         <v>0.25</v>
       </c>
-      <c r="K39" s="17" t="n"/>
+      <c r="K39" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="L39" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M39" s="3" t="inlineStr">
         <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="N39" s="3" t="n"/>
-      <c r="O39" s="3" t="n"/>
-      <c r="P39" s="3" t="n"/>
+      <c r="N39" s="19" t="n">
+        <v>46282</v>
+      </c>
+      <c r="O39" s="19" t="n">
+        <v>46282</v>
+      </c>
+      <c r="P39" s="19" t="n">
+        <v>46282</v>
+      </c>
       <c r="Q39" s="3" t="inlineStr">
         <is>
           <t>asciidoc gone from allowlist and Dockerfile</t>
@@ -4166,12 +4164,12 @@
       </c>
       <c r="R39" s="3" t="inlineStr">
         <is>
-          <t>Blocked on upstream PR</t>
+          <t>Upstream content-core#58 merged 2026-09-05 (v2.1.0); bumped and stripped in this fork</t>
         </is>
       </c>
       <c r="S39" s="3" t="inlineStr">
         <is>
-          <t>content-core#58</t>
+          <t>PR #23; content-core#58; content-core v2.1.0</t>
         </is>
       </c>
     </row>
@@ -6017,7 +6015,7 @@
           <t>docs/SHARING.md; branch ready for PR</t>
         </is>
       </c>
-      <c r="F62" s="25" t="inlineStr">
+      <c r="F62" s="24" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -6101,9 +6099,9 @@
           <t>Entra-backed groups with live membership</t>
         </is>
       </c>
-      <c r="F63" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F63" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G63" s="16" t="inlineStr">
@@ -6146,7 +6144,7 @@
       </c>
       <c r="S63" s="3" t="inlineStr">
         <is>
-          <t>user_group.source / entra_group_oid; docs/SHARING.md</t>
+          <t>user_group.source / entra_group_oid; docs/SHARING.md; api/graph_client.py; commands/entra_group_sync.py</t>
         </is>
       </c>
     </row>
@@ -6163,24 +6161,24 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Full org directory user picker (Graph)</t>
+          <t>Full org directory user picker (Graph) + JIT-stub Entra group members</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Purpose: let owners/admins pick any user in the Entra tenant, not only people who have already signed into the app.
-Why deferred: WP2b picker uses GET /api/users (JIT-provisioned DB rows only) to avoid Graph scopes and pending-grant edge cases.
-Steps: (1) Graph User.Read.All or equivalent search; (2) typeahead against tenant directory; (3) on grant to never-seen user, either JIT stub user or pending grant resolved at first login; (4) document privacy/consent.</t>
+          <t>Purpose: let owners/admins pick any user in the Entra tenant, not only people who have already signed into the app, AND surface Entra group members that have never signed in yet.
+Why deferred (pre-4.21): WP2b picker used GET /api/users (JIT-provisioned DB rows only) to avoid Graph scopes and pending-grant edge cases. WBS 4.20 sync skipped Entra group members with no local user row for the same reason.
+Delivered (PR feat/wbs-4.21-directory-picker): (1) Graph User.Read.All permission documented alongside 4.20's GroupMember.Read.All; (2) GET /api/users/directory tenant-directory typeahead + POST /api/users/from-entra JIT-stub endpoint (both authenticated, not admin-only; from-entra validates the OID against Graph before insert to prevent forgery); (3) commands/entra_group_sync.py now stubs previously-skipped members via list_users_by_oids chunked at 15; (4) upsert-at-first-login already exercised by existing EntraOIDCProvider test; (5) InviteFromDirectoryDialog wired into Groups admin page and ShareSheet, "Never signed in" badge on stub users; (6) AUTH.md § Directory picker + SHARING.md updated; env vars documented (no new env — reuses Entra client credentials).</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Directory-backed share/group member picker</t>
-        </is>
-      </c>
-      <c r="F64" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+          <t>Directory-backed share/group member picker; Entra group members visible before first login</t>
+        </is>
+      </c>
+      <c r="F64" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G64" s="16" t="inlineStr">
@@ -6194,10 +6192,10 @@
         </is>
       </c>
       <c r="I64" s="17" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="J64" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K64" s="17" t="n"/>
       <c r="L64" s="18" t="n">
@@ -6213,17 +6211,17 @@
       <c r="P64" s="3" t="n"/>
       <c r="Q64" s="3" t="inlineStr">
         <is>
-          <t>Can share with a colleague who has never opened the app yet; first login attaches access</t>
+          <t>Admin/owner can share with any tenant colleague (never opened app) + WBS 4.20 sync stops skipping unknown members</t>
         </is>
       </c>
       <c r="R64" s="3" t="inlineStr">
         <is>
-          <t>Pairs with 4.20; keep DB-user picker as fallback</t>
+          <t>Pairs with 4.20; keep DB-user picker as fallback; JIT-stub semantics touch sync + share flow — one spec, one PR</t>
         </is>
       </c>
       <c r="S64" s="3" t="inlineStr">
         <is>
-          <t>GET /api/users today = signed-in only</t>
+          <t>GET /api/users today = signed-in only; entra_group_sync.py members_skipped_unknown counter</t>
         </is>
       </c>
     </row>
@@ -6309,28 +6307,29 @@
     <row r="66" ht="75" customHeight="1">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.23</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>WP3 — Frontend Map + White-label</t>
+          <t>Carry-forward / Sharing Follow-through</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>WP3 kickoff</t>
+          <t>Entra ID group-membership webhooks (Graph change notifications)</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Purpose: start white-label work only after identity is on main.
-Steps: create wp-3-white-label; confirm Model A brand loads once at app startup (not per request).</t>
+          <t>Purpose: replace WBS 4.20's polling loop (default 15 min) with live push-based updates from Microsoft Graph so ACL changes propagate within seconds.
+Why deferred from 4.20: needs a publicly-reachable HTTPS callback URL, HMAC/clientState validation, subscription lifecycle (create + auto-renewal every ~3 days per Graph limit), replay-dedupe, and rotation of the validation token — each with its own security review. Bundling with 4.20 would ~double that PR's risk surface.
+Steps: (1) design spec covering callback URL, clientState secret storage, subscription table schema, renewal cron; (2) POST /api/graph/webhook endpoint with validation-token handshake + subscribe/renew/delete lifecycle; (3) event handler that maps 'groupMembers changed' events to a scoped sync_entra_groups(group_id=...) submission; (4) background job that renews subscriptions with lead time before ~3-day expiry; (5) fall back cleanly to the periodic loop when the webhook subscription is missing or invalid; (6) docs (AUTH.md § Entra group sync/webhooks) + admin UI status pill for subscription health.</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Branch</t>
+          <t>Live push-based Entra group-membership sync</t>
         </is>
       </c>
       <c r="F66" s="22" t="inlineStr">
@@ -6338,21 +6337,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G66" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G66" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>4.19</t>
+          <t>4.20</t>
         </is>
       </c>
       <c r="I66" s="17" t="n">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="J66" s="17" t="n">
-        <v>0.25</v>
+        <v>4</v>
       </c>
       <c r="K66" s="17" t="n"/>
       <c r="L66" s="18" t="n">
@@ -6360,32 +6359,32 @@
       </c>
       <c r="M66" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
-        </is>
-      </c>
-      <c r="N66" s="19" t="n">
-        <v>46253</v>
-      </c>
-      <c r="O66" s="19" t="n">
-        <v>46253</v>
-      </c>
+          <t>Backend Engineer</t>
+        </is>
+      </c>
+      <c r="N66" s="3" t="n"/>
+      <c r="O66" s="3" t="n"/>
       <c r="P66" s="3" t="n"/>
       <c r="Q66" s="3" t="inlineStr">
         <is>
-          <t>Branch created after WP2b merge (or after WP2 if WP2b still open — prefer after 4.19)</t>
+          <t>Entra group membership changes reflect in ACL within seconds (not up to 15 min); subscriptions auto-renew before expiry; missing/invalid subscription silently falls back to the existing periodic loop</t>
         </is>
       </c>
       <c r="R66" s="3" t="inlineStr">
         <is>
-          <t>Optional admin brand UI needs WP2 roles; do not mix with wp-2b-sharing</t>
-        </is>
-      </c>
-      <c r="S66" s="3" t="inlineStr"/>
+          <t>Do NOT bundle with 4.20 — subscription lifecycle deserves its own PR + security review</t>
+        </is>
+      </c>
+      <c r="S66" s="3" t="inlineStr">
+        <is>
+          <t>commands/entra_group_sync.py periodic loop; docs/AUTH.md § Entra group sync (WBS 4.20)</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="75" customHeight="1">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -6395,18 +6394,18 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Produce docs/FRONTEND_MAP.md</t>
+          <t>WP3 kickoff</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Purpose: make every future UI change locatable without archaeology.
-Steps: for each auth and dashboard route, document page → component tree, stores/hooks/API calls, shared layout, component catalog, and a where-do-I-change-X table.</t>
+          <t>Purpose: start white-label work only after identity is on main.
+Steps: create wp-3-white-label; confirm Model A brand loads once at app startup (not per request).</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>docs/FRONTEND_MAP.md</t>
+          <t>Branch</t>
         </is>
       </c>
       <c r="F67" s="22" t="inlineStr">
@@ -6421,14 +6420,14 @@
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.19</t>
         </is>
       </c>
       <c r="I67" s="17" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="J67" s="17" t="n">
-        <v>2.5</v>
+        <v>0.25</v>
       </c>
       <c r="K67" s="17" t="n"/>
       <c r="L67" s="18" t="n">
@@ -6443,21 +6442,25 @@
         <v>46253</v>
       </c>
       <c r="O67" s="19" t="n">
-        <v>46255</v>
+        <v>46253</v>
       </c>
       <c r="P67" s="3" t="n"/>
       <c r="Q67" s="3" t="inlineStr">
         <is>
-          <t>Map covers every route with data flow + backend calls</t>
-        </is>
-      </c>
-      <c r="R67" s="3" t="inlineStr"/>
+          <t>Branch created after WP2b merge (or after WP2 if WP2b still open — prefer after 4.19)</t>
+        </is>
+      </c>
+      <c r="R67" s="3" t="inlineStr">
+        <is>
+          <t>Optional admin brand UI needs WP2 roles; do not mix with wp-2b-sharing</t>
+        </is>
+      </c>
       <c r="S67" s="3" t="inlineStr"/>
     </row>
     <row r="68" ht="75" customHeight="1">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -6467,18 +6470,18 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>BrandConfig schema + loader</t>
+          <t>Produce docs/FRONTEND_MAP.md</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Purpose: drive app name, logos, favicon, colours, font, and support URL from config so clients do not need a rebuild.
-Steps: define BrandConfig schema; load from BRAND_CONFIG_PATH or /config/brand at startup under Model A.</t>
+          <t>Purpose: make every future UI change locatable without archaeology.
+Steps: for each auth and dashboard route, document page → component tree, stores/hooks/API calls, shared layout, component catalog, and a where-do-I-change-X table.</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>BrandConfig type + loader</t>
+          <t>docs/FRONTEND_MAP.md</t>
         </is>
       </c>
       <c r="F68" s="22" t="inlineStr">
@@ -6486,9 +6489,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G68" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G68" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr">
@@ -6497,10 +6500,10 @@
         </is>
       </c>
       <c r="I68" s="17" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="J68" s="17" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="K68" s="17" t="n"/>
       <c r="L68" s="18" t="n">
@@ -6508,19 +6511,19 @@
       </c>
       <c r="M68" s="3" t="inlineStr">
         <is>
-          <t>Full-stack</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N68" s="19" t="n">
+        <v>46253</v>
+      </c>
+      <c r="O68" s="19" t="n">
         <v>46255</v>
-      </c>
-      <c r="O68" s="19" t="n">
-        <v>46256</v>
       </c>
       <c r="P68" s="3" t="n"/>
       <c r="Q68" s="3" t="inlineStr">
         <is>
-          <t>Config loads without a rebuild</t>
+          <t>Map covers every route with data flow + backend calls</t>
         </is>
       </c>
       <c r="R68" s="3" t="inlineStr"/>
@@ -6529,7 +6532,7 @@
     <row r="69" ht="75" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>5.2</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -6539,18 +6542,18 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Runtime theme injection (CSS variables)</t>
+          <t>BrandConfig schema + loader</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Purpose: apply BrandConfig at runtime to CSS variables for light and dark themes.
-Steps: map colours to :root / dark variants; replace hardcoded title and /logo.svg; use the brand inventory in LICENSE_COMPLIANCE §8; demonstrate two brands from one build.</t>
+          <t>Purpose: drive app name, logos, favicon, colours, font, and support URL from config so clients do not need a rebuild.
+Steps: define BrandConfig schema; load from BRAND_CONFIG_PATH or /config/brand at startup under Model A.</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Runtime theming</t>
+          <t>BrandConfig type + loader</t>
         </is>
       </c>
       <c r="F69" s="22" t="inlineStr">
@@ -6565,14 +6568,14 @@
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="I69" s="17" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="J69" s="17" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="K69" s="17" t="n"/>
       <c r="L69" s="18" t="n">
@@ -6580,19 +6583,19 @@
       </c>
       <c r="M69" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>Full-stack</t>
         </is>
       </c>
       <c r="N69" s="19" t="n">
+        <v>46255</v>
+      </c>
+      <c r="O69" s="19" t="n">
         <v>46256</v>
-      </c>
-      <c r="O69" s="19" t="n">
-        <v>46259</v>
       </c>
       <c r="P69" s="3" t="n"/>
       <c r="Q69" s="3" t="inlineStr">
         <is>
-          <t>Two visibly different brands from the same build; no code edit to rebrand</t>
+          <t>Config loads without a rebuild</t>
         </is>
       </c>
       <c r="R69" s="3" t="inlineStr"/>
@@ -6601,7 +6604,7 @@
     <row r="70" ht="75" customHeight="1">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>5.4</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -6611,18 +6614,18 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>themes/ presets + add-client procedure</t>
+          <t>Runtime theme injection (CSS variables)</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Purpose: make “add a client theme” a documented drop-in of config + assets.
-Steps: ship at least two presets under themes/; write the operator procedure (no rebuild).</t>
+          <t>Purpose: apply BrandConfig at runtime to CSS variables for light and dark themes.
+Steps: map colours to :root / dark variants; replace hardcoded title and /logo.svg; use the brand inventory in LICENSE_COMPLIANCE §8; demonstrate two brands from one build.</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>themes/ + docs procedure</t>
+          <t>Runtime theming</t>
         </is>
       </c>
       <c r="F70" s="22" t="inlineStr">
@@ -6630,21 +6633,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G70" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G70" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>5.2</t>
         </is>
       </c>
       <c r="I70" s="17" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="J70" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K70" s="17" t="n"/>
       <c r="L70" s="18" t="n">
@@ -6656,15 +6659,15 @@
         </is>
       </c>
       <c r="N70" s="19" t="n">
+        <v>46256</v>
+      </c>
+      <c r="O70" s="19" t="n">
         <v>46259</v>
-      </c>
-      <c r="O70" s="19" t="n">
-        <v>46260</v>
       </c>
       <c r="P70" s="3" t="n"/>
       <c r="Q70" s="3" t="inlineStr">
         <is>
-          <t>Documented procedure produces two different brands from one build</t>
+          <t>Two visibly different brands from the same build; no code edit to rebrand</t>
         </is>
       </c>
       <c r="R70" s="3" t="inlineStr"/>
@@ -6673,7 +6676,7 @@
     <row r="71" ht="75" customHeight="1">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -6683,18 +6686,18 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Optional admin BrandConfig UI</t>
+          <t>themes/ presets + add-client procedure</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Purpose (optional): let admins edit BrandConfig live without redeploying.
-Steps: admin-only settings screen gated by WP2 roles; persist and hot-apply theme.</t>
+          <t>Purpose: make “add a client theme” a documented drop-in of config + assets.
+Steps: ship at least two presets under themes/; write the operator procedure (no rebuild).</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Admin brand settings UI</t>
+          <t>themes/ + docs procedure</t>
         </is>
       </c>
       <c r="F71" s="22" t="inlineStr">
@@ -6702,21 +6705,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G71" s="24" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="G71" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>5.3,4.5</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="I71" s="17" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="J71" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K71" s="17" t="n"/>
       <c r="L71" s="18" t="n">
@@ -6728,28 +6731,24 @@
         </is>
       </c>
       <c r="N71" s="19" t="n">
+        <v>46259</v>
+      </c>
+      <c r="O71" s="19" t="n">
         <v>46260</v>
-      </c>
-      <c r="O71" s="19" t="n">
-        <v>46262</v>
       </c>
       <c r="P71" s="3" t="n"/>
       <c r="Q71" s="3" t="inlineStr">
         <is>
-          <t>Admin can edit brand without redeploy (optional acceptance)</t>
-        </is>
-      </c>
-      <c r="R71" s="3" t="inlineStr">
-        <is>
-          <t>Optional per master plan</t>
-        </is>
-      </c>
+          <t>Documented procedure produces two different brands from one build</t>
+        </is>
+      </c>
+      <c r="R71" s="3" t="inlineStr"/>
       <c r="S71" s="3" t="inlineStr"/>
     </row>
     <row r="72" ht="75" customHeight="1">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -6759,18 +6758,18 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>WP3 verification + review stop</t>
+          <t>Optional admin BrandConfig UI</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Purpose: close white-label only when map + config branding acceptance criteria pass.
-Steps: verify ACs; PR; human review; do not mix WP5 on the same branch.</t>
+          <t>Purpose (optional): let admins edit BrandConfig live without redeploying.
+Steps: admin-only settings screen gated by WP2 roles; persist and hot-apply theme.</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>Merged WP3</t>
+          <t>Admin brand settings UI</t>
         </is>
       </c>
       <c r="F72" s="22" t="inlineStr">
@@ -6778,21 +6777,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G72" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G72" s="23" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>5.1,5.4</t>
+          <t>5.3,4.5</t>
         </is>
       </c>
       <c r="I72" s="17" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="J72" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K72" s="17" t="n"/>
       <c r="L72" s="18" t="n">
@@ -6800,49 +6799,53 @@
       </c>
       <c r="M72" s="3" t="inlineStr">
         <is>
-          <t>Engineering Lead</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N72" s="19" t="n">
+        <v>46260</v>
+      </c>
+      <c r="O72" s="19" t="n">
         <v>46262</v>
-      </c>
-      <c r="O72" s="19" t="n">
-        <v>46263</v>
       </c>
       <c r="P72" s="3" t="n"/>
       <c r="Q72" s="3" t="inlineStr">
         <is>
-          <t>All WP3 acceptance criteria pass</t>
-        </is>
-      </c>
-      <c r="R72" s="3" t="inlineStr"/>
+          <t>Admin can edit brand without redeploy (optional acceptance)</t>
+        </is>
+      </c>
+      <c r="R72" s="3" t="inlineStr">
+        <is>
+          <t>Optional per master plan</t>
+        </is>
+      </c>
       <c r="S72" s="3" t="inlineStr"/>
     </row>
     <row r="73" ht="75" customHeight="1">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>WP4 — Backend/API Documentation</t>
+          <t>WP3 — Frontend Map + White-label</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>WP4 kickoff (can parallel early)</t>
+          <t>WP3 verification + review stop</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Purpose: start the backend architecture map as documentation-only, low-risk work.
-Steps: create wp-4-backend-map; prefer starting after WP2 so auth docs match reality; can begin after WP0 if staffed in parallel.</t>
+          <t>Purpose: close white-label only when map + config branding acceptance criteria pass.
+Steps: verify ACs; PR; human review; do not mix WP5 on the same branch.</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Branch</t>
+          <t>Merged WP3</t>
         </is>
       </c>
       <c r="F73" s="22" t="inlineStr">
@@ -6850,21 +6853,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G73" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G73" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>5.1,5.4</t>
         </is>
       </c>
       <c r="I73" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="J73" s="17" t="n">
         <v>1</v>
-      </c>
-      <c r="J73" s="17" t="n">
-        <v>0.25</v>
       </c>
       <c r="K73" s="17" t="n"/>
       <c r="L73" s="18" t="n">
@@ -6872,439 +6875,475 @@
       </c>
       <c r="M73" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Engineering Lead</t>
         </is>
       </c>
       <c r="N73" s="19" t="n">
-        <v>46253</v>
+        <v>46262</v>
       </c>
       <c r="O73" s="19" t="n">
-        <v>46253</v>
+        <v>46263</v>
       </c>
       <c r="P73" s="3" t="n"/>
       <c r="Q73" s="3" t="inlineStr">
         <is>
-          <t>Docs branch ready</t>
-        </is>
-      </c>
-      <c r="R73" s="3" t="inlineStr">
-        <is>
-          <t>Better after WP2 for accurate auth sections</t>
-        </is>
-      </c>
+          <t>All WP3 acceptance criteria pass</t>
+        </is>
+      </c>
+      <c r="R73" s="3" t="inlineStr"/>
       <c r="S73" s="3" t="inlineStr"/>
     </row>
     <row r="74" ht="75" customHeight="1">
       <c r="A74" s="3" t="inlineStr">
         <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>WP4 — Backend/API Documentation</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>WP4 kickoff (can parallel early)</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: start the backend architecture map as documentation-only, low-risk work.
+Steps: create wp-4-backend-map; prefer starting after WP2 so auth docs match reality; can begin after WP0 if staffed in parallel.</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="F74" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G74" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>1.11</t>
+        </is>
+      </c>
+      <c r="I74" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J74" s="17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K74" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L74" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M74" s="3" t="inlineStr">
+        <is>
+          <t>Backend Engineer</t>
+        </is>
+      </c>
+      <c r="N74" s="19" t="n">
+        <v>46253</v>
+      </c>
+      <c r="O74" s="19" t="n">
+        <v>46253</v>
+      </c>
+      <c r="P74" s="19" t="n">
+        <v>46294</v>
+      </c>
+      <c r="Q74" s="3" t="inlineStr">
+        <is>
+          <t>Docs branch ready</t>
+        </is>
+      </c>
+      <c r="R74" s="3" t="inlineStr">
+        <is>
+          <t>Better after WP2 for accurate auth sections</t>
+        </is>
+      </c>
+      <c r="S74" s="3" t="inlineStr">
+        <is>
+          <t>PR #55</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="75" customHeight="1">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
           <t>6.1</t>
         </is>
       </c>
-      <c r="B74" s="3" t="inlineStr">
+      <c r="B75" s="3" t="inlineStr">
         <is>
           <t>WP4 — Backend/API Documentation</t>
         </is>
       </c>
-      <c r="C74" s="3" t="inlineStr">
+      <c r="C75" s="3" t="inlineStr">
         <is>
           <t>Router catalog (all endpoints)</t>
         </is>
       </c>
-      <c r="D74" s="3" t="inlineStr">
+      <c r="D75" s="3" t="inlineStr">
         <is>
           <t>Purpose: catalogue every HTTP endpoint with method, path, models, auth requirement, and service/domain call.
 Steps: walk all routers; document consistently; update after WP2 auth lands.</t>
         </is>
       </c>
-      <c r="E74" s="3" t="inlineStr">
+      <c r="E75" s="3" t="inlineStr">
         <is>
           <t>BACKEND_MAP.md routers section</t>
         </is>
       </c>
-      <c r="F74" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G74" s="21" t="inlineStr">
+      <c r="F75" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G75" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H74" s="3" t="inlineStr">
+      <c r="H75" s="3" t="inlineStr">
         <is>
           <t>6.0</t>
         </is>
       </c>
-      <c r="I74" s="17" t="n">
+      <c r="I75" s="17" t="n">
         <v>16</v>
       </c>
-      <c r="J74" s="17" t="n">
+      <c r="J75" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="K74" s="17" t="n"/>
-      <c r="L74" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M74" s="3" t="inlineStr">
+      <c r="K75" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="L75" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M75" s="3" t="inlineStr">
         <is>
           <t>Backend Engineer</t>
         </is>
       </c>
-      <c r="N74" s="19" t="n">
+      <c r="N75" s="19" t="n">
         <v>46253</v>
       </c>
-      <c r="O74" s="19" t="n">
+      <c r="O75" s="19" t="n">
         <v>46255</v>
       </c>
-      <c r="P74" s="3" t="n"/>
-      <c r="Q74" s="3" t="inlineStr">
+      <c r="P75" s="19" t="n">
+        <v>46294</v>
+      </c>
+      <c r="Q75" s="3" t="inlineStr">
         <is>
           <t>Every endpoint documented with auth + models</t>
         </is>
       </c>
-      <c r="R74" s="3" t="inlineStr"/>
-      <c r="S74" s="3" t="inlineStr"/>
-    </row>
-    <row r="75" ht="75" customHeight="1">
-      <c r="A75" s="3" t="inlineStr">
+      <c r="R75" s="3" t="inlineStr"/>
+      <c r="S75" s="3" t="inlineStr">
+        <is>
+          <t>PR #55 docs/BACKEND_MAP.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="75" customHeight="1">
+      <c r="A76" s="3" t="inlineStr">
         <is>
           <t>6.2</t>
         </is>
       </c>
-      <c r="B75" s="3" t="inlineStr">
+      <c r="B76" s="3" t="inlineStr">
         <is>
           <t>WP4 — Backend/API Documentation</t>
         </is>
       </c>
-      <c r="C75" s="3" t="inlineStr">
+      <c r="C76" s="3" t="inlineStr">
         <is>
           <t>Domain model + graph + data layer maps</t>
         </is>
       </c>
-      <c r="D75" s="3" t="inlineStr">
+      <c r="D76" s="3" t="inlineStr">
         <is>
           <t>Purpose: document ObjectModel patterns, LangGraph flows, repository usage, migrations, and SurrealDB features in use.
 Steps: catalogue models/relationships; map each graph’s inputs/steps/outputs; explain repository call-site pattern and migrations.</t>
         </is>
       </c>
-      <c r="E75" s="3" t="inlineStr">
+      <c r="E76" s="3" t="inlineStr">
         <is>
           <t>BACKEND_MAP.md domain/graphs/data</t>
         </is>
       </c>
-      <c r="F75" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G75" s="21" t="inlineStr">
+      <c r="F76" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G76" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H75" s="3" t="inlineStr">
+      <c r="H76" s="3" t="inlineStr">
         <is>
           <t>6.1</t>
         </is>
       </c>
-      <c r="I75" s="17" t="n">
+      <c r="I76" s="17" t="n">
         <v>16</v>
       </c>
-      <c r="J75" s="17" t="n">
+      <c r="J76" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="K75" s="17" t="n"/>
-      <c r="L75" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M75" s="3" t="inlineStr">
+      <c r="K76" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="L76" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M76" s="3" t="inlineStr">
         <is>
           <t>Backend Engineer</t>
         </is>
       </c>
-      <c r="N75" s="19" t="n">
+      <c r="N76" s="19" t="n">
         <v>46255</v>
       </c>
-      <c r="O75" s="19" t="n">
+      <c r="O76" s="19" t="n">
         <v>46259</v>
       </c>
-      <c r="P75" s="3" t="n"/>
-      <c r="Q75" s="3" t="inlineStr">
+      <c r="P76" s="19" t="n">
+        <v>46294</v>
+      </c>
+      <c r="Q76" s="3" t="inlineStr">
         <is>
           <t>Every domain model and graph documented</t>
         </is>
       </c>
-      <c r="R75" s="3" t="inlineStr"/>
-      <c r="S75" s="3" t="inlineStr"/>
-    </row>
-    <row r="76" ht="75" customHeight="1">
-      <c r="A76" s="3" t="inlineStr">
+      <c r="R76" s="3" t="inlineStr"/>
+      <c r="S76" s="3" t="inlineStr">
+        <is>
+          <t>PR #55 docs/BACKEND_MAP.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="75" customHeight="1">
+      <c r="A77" s="3" t="inlineStr">
         <is>
           <t>6.3</t>
         </is>
       </c>
-      <c r="B76" s="3" t="inlineStr">
+      <c r="B77" s="3" t="inlineStr">
         <is>
           <t>WP4 — Backend/API Documentation</t>
         </is>
       </c>
-      <c r="C76" s="3" t="inlineStr">
+      <c r="C77" s="3" t="inlineStr">
         <is>
           <t>Jobs, config/secrets, how-to playbooks</t>
         </is>
       </c>
-      <c r="D76" s="3" t="inlineStr">
+      <c r="D77" s="3" t="inlineStr">
         <is>
           <t>Purpose: finish the operator/engineer map with jobs, env vars, and five how-to-add playbooks.
 Steps: document surreal-commands; env/secrets; playbooks for endpoint, model+migration, provider, job, source type; reconcile with existing change-playbooks.md.</t>
         </is>
       </c>
-      <c r="E76" s="3" t="inlineStr">
+      <c r="E77" s="3" t="inlineStr">
         <is>
           <t>BACKEND_MAP.md complete</t>
         </is>
       </c>
-      <c r="F76" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G76" s="21" t="inlineStr">
+      <c r="F77" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G77" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H76" s="3" t="inlineStr">
+      <c r="H77" s="3" t="inlineStr">
         <is>
           <t>6.2</t>
         </is>
       </c>
-      <c r="I76" s="17" t="n">
+      <c r="I77" s="17" t="n">
         <v>12</v>
       </c>
-      <c r="J76" s="17" t="n">
+      <c r="J77" s="17" t="n">
         <v>1.5</v>
       </c>
-      <c r="K76" s="17" t="n"/>
-      <c r="L76" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M76" s="3" t="inlineStr">
+      <c r="K77" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="L77" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M77" s="3" t="inlineStr">
         <is>
           <t>Backend Engineer</t>
         </is>
       </c>
-      <c r="N76" s="19" t="n">
+      <c r="N77" s="19" t="n">
         <v>46259</v>
       </c>
-      <c r="O76" s="19" t="n">
+      <c r="O77" s="19" t="n">
         <v>46260</v>
       </c>
-      <c r="P76" s="3" t="n"/>
-      <c r="Q76" s="3" t="inlineStr">
+      <c r="P77" s="19" t="n">
+        <v>46294</v>
+      </c>
+      <c r="Q77" s="3" t="inlineStr">
         <is>
           <t>Five how-to playbooks present and accurate</t>
         </is>
       </c>
-      <c r="R76" s="3" t="inlineStr"/>
-      <c r="S76" s="3" t="inlineStr"/>
-    </row>
-    <row r="77" ht="75" customHeight="1">
-      <c r="A77" s="3" t="inlineStr">
+      <c r="R77" s="3" t="inlineStr"/>
+      <c r="S77" s="3" t="inlineStr">
+        <is>
+          <t>PR #55 docs/BACKEND_MAP.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="75" customHeight="1">
+      <c r="A78" s="3" t="inlineStr">
         <is>
           <t>6.4</t>
         </is>
       </c>
-      <c r="B77" s="3" t="inlineStr">
+      <c r="B78" s="3" t="inlineStr">
         <is>
           <t>WP4 — Backend/API Documentation</t>
         </is>
       </c>
-      <c r="C77" s="3" t="inlineStr">
+      <c r="C78" s="3" t="inlineStr">
         <is>
           <t>WP4 review stop</t>
         </is>
       </c>
-      <c r="D77" s="3" t="inlineStr">
+      <c r="D78" s="3" t="inlineStr">
         <is>
           <t>Purpose: peer-review the map for accuracy and merge.
 Steps: review against live code; fix gaps; merge; confirm a new engineer can locate changes using only BACKEND_MAP.</t>
         </is>
       </c>
-      <c r="E77" s="3" t="inlineStr">
+      <c r="E78" s="3" t="inlineStr">
         <is>
           <t>docs/BACKEND_MAP.md on main</t>
         </is>
       </c>
-      <c r="F77" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G77" s="21" t="inlineStr">
+      <c r="F78" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G78" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H77" s="3" t="inlineStr">
+      <c r="H78" s="3" t="inlineStr">
         <is>
           <t>6.3</t>
         </is>
       </c>
-      <c r="I77" s="17" t="n">
+      <c r="I78" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="J77" s="17" t="n">
+      <c r="J78" s="17" t="n">
         <v>0.5</v>
       </c>
-      <c r="K77" s="17" t="n"/>
-      <c r="L77" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M77" s="3" t="inlineStr">
+      <c r="K78" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="L78" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M78" s="3" t="inlineStr">
         <is>
           <t>Engineering Lead</t>
         </is>
       </c>
-      <c r="N77" s="19" t="n">
+      <c r="N78" s="19" t="n">
         <v>46260</v>
       </c>
-      <c r="O77" s="19" t="n">
+      <c r="O78" s="19" t="n">
         <v>46261</v>
       </c>
-      <c r="P77" s="3" t="n"/>
-      <c r="Q77" s="3" t="inlineStr">
+      <c r="P78" s="19" t="n">
+        <v>46294</v>
+      </c>
+      <c r="Q78" s="3" t="inlineStr">
         <is>
           <t>New engineer can locate changes using only this doc</t>
         </is>
       </c>
-      <c r="R77" s="3" t="inlineStr"/>
-      <c r="S77" s="3" t="inlineStr"/>
-    </row>
-    <row r="78" ht="75" customHeight="1">
-      <c r="A78" s="3" t="inlineStr">
+      <c r="R78" s="3" t="inlineStr"/>
+      <c r="S78" s="3" t="inlineStr">
+        <is>
+          <t>PR #55</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="75" customHeight="1">
+      <c r="A79" s="3" t="inlineStr">
         <is>
           <t>7.0</t>
         </is>
       </c>
-      <c r="B78" s="3" t="inlineStr">
+      <c r="B79" s="3" t="inlineStr">
         <is>
           <t>WP5 — External Source Connectors</t>
         </is>
       </c>
-      <c r="C78" s="3" t="inlineStr">
+      <c r="C79" s="3" t="inlineStr">
         <is>
           <t>WP5 kickoff</t>
         </is>
       </c>
-      <c r="D78" s="3" t="inlineStr">
+      <c r="D79" s="3" t="inlineStr">
         <is>
           <t>Purpose: design connectors that feed the existing ingestion pipeline instead of reinventing extraction.
 Steps: create wp-5-connectors; draft SourceConnector interface; confirm hard dependency on WP2 for per-user OAuth tokens.</t>
         </is>
       </c>
-      <c r="E78" s="3" t="inlineStr">
+      <c r="E79" s="3" t="inlineStr">
         <is>
           <t>Branch + design note</t>
         </is>
       </c>
-      <c r="F78" s="22" t="inlineStr">
+      <c r="F79" s="22" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G78" s="16" t="inlineStr">
+      <c r="G79" s="16" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H78" s="3" t="inlineStr">
+      <c r="H79" s="3" t="inlineStr">
         <is>
           <t>4.10</t>
         </is>
       </c>
-      <c r="I78" s="17" t="n">
+      <c r="I79" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="J78" s="17" t="n">
+      <c r="J79" s="17" t="n">
         <v>0.5</v>
-      </c>
-      <c r="K78" s="17" t="n"/>
-      <c r="L78" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M78" s="3" t="inlineStr">
-        <is>
-          <t>Engineer</t>
-        </is>
-      </c>
-      <c r="N78" s="19" t="n">
-        <v>46266</v>
-      </c>
-      <c r="O78" s="19" t="n">
-        <v>46266</v>
-      </c>
-      <c r="P78" s="3" t="n"/>
-      <c r="Q78" s="3" t="inlineStr">
-        <is>
-          <t>Design reuses content-core + graphs/source.py</t>
-        </is>
-      </c>
-      <c r="R78" s="3" t="inlineStr">
-        <is>
-          <t>Blocked until WP2 users/tokens exist</t>
-        </is>
-      </c>
-      <c r="S78" s="3" t="inlineStr"/>
-    </row>
-    <row r="79" ht="75" customHeight="1">
-      <c r="A79" s="3" t="inlineStr">
-        <is>
-          <t>7.1</t>
-        </is>
-      </c>
-      <c r="B79" s="3" t="inlineStr">
-        <is>
-          <t>WP5 — External Source Connectors</t>
-        </is>
-      </c>
-      <c r="C79" s="3" t="inlineStr">
-        <is>
-          <t>SourceConnector interface + bulk job fan-out</t>
-        </is>
-      </c>
-      <c r="D79" s="3" t="inlineStr">
-        <is>
-          <t>Purpose: one “add location” action becomes N document jobs with per-doc progress and partial failure tolerance.
-Steps: define authenticate/list_documents/fetch_document; extend source_commands for fan-out; ensure one bad file does not abort the batch.</t>
-        </is>
-      </c>
-      <c r="E79" s="3" t="inlineStr">
-        <is>
-          <t>Connector API + bulk command</t>
-        </is>
-      </c>
-      <c r="F79" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G79" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="H79" s="3" t="inlineStr">
-        <is>
-          <t>7.0</t>
-        </is>
-      </c>
-      <c r="I79" s="17" t="n">
-        <v>24</v>
-      </c>
-      <c r="J79" s="17" t="n">
-        <v>3</v>
       </c>
       <c r="K79" s="17" t="n"/>
       <c r="L79" s="18" t="n">
@@ -7312,28 +7351,32 @@
       </c>
       <c r="M79" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N79" s="19" t="n">
         <v>46266</v>
       </c>
       <c r="O79" s="19" t="n">
-        <v>46269</v>
+        <v>46266</v>
       </c>
       <c r="P79" s="3" t="n"/>
       <c r="Q79" s="3" t="inlineStr">
         <is>
-          <t>Single failure does not abort batch; progress per document</t>
-        </is>
-      </c>
-      <c r="R79" s="3" t="inlineStr"/>
+          <t>Design reuses content-core + graphs/source.py</t>
+        </is>
+      </c>
+      <c r="R79" s="3" t="inlineStr">
+        <is>
+          <t>Blocked until WP2 users/tokens exist</t>
+        </is>
+      </c>
       <c r="S79" s="3" t="inlineStr"/>
     </row>
     <row r="80" ht="75" customHeight="1">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
@@ -7343,18 +7386,18 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>SharePoint connector (Microsoft Graph)</t>
+          <t>SourceConnector interface + bulk job fan-out</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Purpose: let an Entra-signed-in user pull an entire SharePoint folder into chat-able sources.
-Steps: OAuth on behalf of the user; least-privilege Sites/Files read scopes; enumerate folder; download supported files into existing ingestion; document admin consent.</t>
+          <t>Purpose: one “add location” action becomes N document jobs with per-doc progress and partial failure tolerance.
+Steps: define authenticate/list_documents/fetch_document; extend source_commands for fan-out; ensure one bad file does not abort the batch.</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>SharePointConnector</t>
+          <t>Connector API + bulk command</t>
         </is>
       </c>
       <c r="F80" s="22" t="inlineStr">
@@ -7369,14 +7412,14 @@
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>7.1,4.7</t>
+          <t>7.0</t>
         </is>
       </c>
       <c r="I80" s="17" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="J80" s="17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K80" s="17" t="n"/>
       <c r="L80" s="18" t="n">
@@ -7388,15 +7431,15 @@
         </is>
       </c>
       <c r="N80" s="19" t="n">
+        <v>46266</v>
+      </c>
+      <c r="O80" s="19" t="n">
         <v>46269</v>
-      </c>
-      <c r="O80" s="19" t="n">
-        <v>46275</v>
       </c>
       <c r="P80" s="3" t="n"/>
       <c r="Q80" s="3" t="inlineStr">
         <is>
-          <t>User connects SharePoint, picks folder, pulls all supported docs</t>
+          <t>Single failure does not abort batch; progress per document</t>
         </is>
       </c>
       <c r="R80" s="3" t="inlineStr"/>
@@ -7405,7 +7448,7 @@
     <row r="81" ht="75" customHeight="1">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>7.2</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -7415,18 +7458,18 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Generic DMS / multi-doc link connector</t>
+          <t>SharePoint connector (Microsoft Graph)</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Purpose: support folder URLs / IDs that resolve to many documents, with an extension point for other DMS systems.
-Steps: implement base multi-doc connector; keep the SourceConnector interface as the only required surface for new connectors.</t>
+          <t>Purpose: let an Entra-signed-in user pull an entire SharePoint folder into chat-able sources.
+Steps: OAuth on behalf of the user; least-privilege Sites/Files read scopes; enumerate folder; download supported files into existing ingestion; document admin consent.</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>Generic multi-doc connector</t>
+          <t>SharePointConnector</t>
         </is>
       </c>
       <c r="F81" s="22" t="inlineStr">
@@ -7434,21 +7477,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G81" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G81" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>7.1,4.7</t>
         </is>
       </c>
       <c r="I81" s="17" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="J81" s="17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K81" s="17" t="n"/>
       <c r="L81" s="18" t="n">
@@ -7460,7 +7503,7 @@
         </is>
       </c>
       <c r="N81" s="19" t="n">
-        <v>46273</v>
+        <v>46269</v>
       </c>
       <c r="O81" s="19" t="n">
         <v>46275</v>
@@ -7468,7 +7511,7 @@
       <c r="P81" s="3" t="n"/>
       <c r="Q81" s="3" t="inlineStr">
         <is>
-          <t>New connector = implement interface only</t>
+          <t>User connects SharePoint, picks folder, pulls all supported docs</t>
         </is>
       </c>
       <c r="R81" s="3" t="inlineStr"/>
@@ -7477,7 +7520,7 @@
     <row r="82" ht="75" customHeight="1">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>7.4</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -7487,18 +7530,18 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Encrypted per-user token storage</t>
+          <t>Generic DMS / multi-doc link connector</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Purpose: store connector OAuth tokens encrypted per user using existing encryption-key infrastructure.
-Steps: persist tokens encrypted; never share across users; respect source-system permissions (never fetch what the user cannot access).</t>
+          <t>Purpose: support folder URLs / IDs that resolve to many documents, with an extension point for other DMS systems.
+Steps: implement base multi-doc connector; keep the SourceConnector interface as the only required surface for new connectors.</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>Encrypted token store</t>
+          <t>Generic multi-doc connector</t>
         </is>
       </c>
       <c r="F82" s="22" t="inlineStr">
@@ -7506,21 +7549,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G82" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G82" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>7.2,2.8</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="I82" s="17" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="J82" s="17" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="K82" s="17" t="n"/>
       <c r="L82" s="18" t="n">
@@ -7532,15 +7575,15 @@
         </is>
       </c>
       <c r="N82" s="19" t="n">
+        <v>46273</v>
+      </c>
+      <c r="O82" s="19" t="n">
         <v>46275</v>
-      </c>
-      <c r="O82" s="19" t="n">
-        <v>46276</v>
       </c>
       <c r="P82" s="3" t="n"/>
       <c r="Q82" s="3" t="inlineStr">
         <is>
-          <t>Tokens encrypted per user; no cross-user leak</t>
+          <t>New connector = implement interface only</t>
         </is>
       </c>
       <c r="R82" s="3" t="inlineStr"/>
@@ -7549,7 +7592,7 @@
     <row r="83" ht="75" customHeight="1">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>7.4</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -7559,18 +7602,18 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Frontend: Add from SharePoint / Link flow</t>
+          <t>Encrypted per-user token storage</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Purpose: ship the operator UX for connect → folder pick → select → progress, then chat across the pulled set.
-Steps: add sources steps UI; show per-doc progress; ensure i18n for all locales; group pulled docs for chat/search.</t>
+          <t>Purpose: store connector OAuth tokens encrypted per user using existing encryption-key infrastructure.
+Steps: persist tokens encrypted; never share across users; respect source-system permissions (never fetch what the user cannot access).</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>Sources UI flow</t>
+          <t>Encrypted token store</t>
         </is>
       </c>
       <c r="F83" s="22" t="inlineStr">
@@ -7578,21 +7621,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G83" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G83" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>7.2,7.3</t>
+          <t>7.2,2.8</t>
         </is>
       </c>
       <c r="I83" s="17" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="J83" s="17" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="K83" s="17" t="n"/>
       <c r="L83" s="18" t="n">
@@ -7600,32 +7643,28 @@
       </c>
       <c r="M83" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N83" s="19" t="n">
+        <v>46275</v>
+      </c>
+      <c r="O83" s="19" t="n">
         <v>46276</v>
-      </c>
-      <c r="O83" s="19" t="n">
-        <v>46281</v>
       </c>
       <c r="P83" s="3" t="n"/>
       <c r="Q83" s="3" t="inlineStr">
         <is>
-          <t>User can chat across the whole pulled set</t>
-        </is>
-      </c>
-      <c r="R83" s="3" t="inlineStr">
-        <is>
-          <t>i18n required for all locales</t>
-        </is>
-      </c>
+          <t>Tokens encrypted per user; no cross-user leak</t>
+        </is>
+      </c>
+      <c r="R83" s="3" t="inlineStr"/>
       <c r="S83" s="3" t="inlineStr"/>
     </row>
     <row r="84" ht="75" customHeight="1">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>7.6</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -7635,18 +7674,18 @@
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>docs/CONNECTORS.md + WP5 review</t>
+          <t>Frontend: Add from SharePoint / Link flow</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Purpose: document Entra scopes/consent and how to add a connector; close WP5 on acceptance criteria.
-Steps: write CONNECTORS.md; verify ACs; PR; human review stop.</t>
+          <t>Purpose: ship the operator UX for connect → folder pick → select → progress, then chat across the pulled set.
+Steps: add sources steps UI; show per-doc progress; ensure i18n for all locales; group pulled docs for chat/search.</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>docs/CONNECTORS.md; merged WP5</t>
+          <t>Sources UI flow</t>
         </is>
       </c>
       <c r="F84" s="22" t="inlineStr">
@@ -7661,14 +7700,14 @@
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>7.4,7.5</t>
+          <t>7.2,7.3</t>
         </is>
       </c>
       <c r="I84" s="17" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="J84" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K84" s="17" t="n"/>
       <c r="L84" s="18" t="n">
@@ -7676,49 +7715,53 @@
       </c>
       <c r="M84" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N84" s="19" t="n">
+        <v>46276</v>
+      </c>
+      <c r="O84" s="19" t="n">
         <v>46281</v>
-      </c>
-      <c r="O84" s="19" t="n">
-        <v>46282</v>
       </c>
       <c r="P84" s="3" t="n"/>
       <c r="Q84" s="3" t="inlineStr">
         <is>
-          <t>All WP5 acceptance criteria pass</t>
-        </is>
-      </c>
-      <c r="R84" s="3" t="inlineStr"/>
+          <t>User can chat across the whole pulled set</t>
+        </is>
+      </c>
+      <c r="R84" s="3" t="inlineStr">
+        <is>
+          <t>i18n required for all locales</t>
+        </is>
+      </c>
       <c r="S84" s="3" t="inlineStr"/>
     </row>
     <row r="85" ht="75" customHeight="1">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>7.6</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>WP6 — Doc Processing Benchmarks</t>
+          <t>WP5 — External Source Connectors</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>WP6 kickoff + enumerate supported types</t>
+          <t>docs/CONNECTORS.md + WP5 review</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Purpose: list what content-core actually supports today and what needs work (OCR, EPUB, upload HTML, etc.).
-Steps: inventory from real code/config; note gaps; create wp-6-benchmarks. Can run after WP0; needs target hardware for later measurement tasks.</t>
+          <t>Purpose: document Entra scopes/consent and how to add a connector; close WP5 on acceptance criteria.
+Steps: write CONNECTORS.md; verify ACs; PR; human review stop.</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Type inventory</t>
+          <t>docs/CONNECTORS.md; merged WP5</t>
         </is>
       </c>
       <c r="F85" s="22" t="inlineStr">
@@ -7726,14 +7769,14 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G85" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G85" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>7.4,7.5</t>
         </is>
       </c>
       <c r="I85" s="17" t="n">
@@ -7752,28 +7795,24 @@
         </is>
       </c>
       <c r="N85" s="19" t="n">
-        <v>46266</v>
+        <v>46281</v>
       </c>
       <c r="O85" s="19" t="n">
-        <v>46267</v>
+        <v>46282</v>
       </c>
       <c r="P85" s="3" t="n"/>
       <c r="Q85" s="3" t="inlineStr">
         <is>
-          <t>Supported types documented from real code</t>
-        </is>
-      </c>
-      <c r="R85" s="3" t="inlineStr">
-        <is>
-          <t>No guessed client-facing numbers</t>
-        </is>
-      </c>
+          <t>All WP5 acceptance criteria pass</t>
+        </is>
+      </c>
+      <c r="R85" s="3" t="inlineStr"/>
       <c r="S85" s="3" t="inlineStr"/>
     </row>
     <row r="86" ht="75" customHeight="1">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -7783,18 +7822,18 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Build /benchmarks/ harness</t>
+          <t>WP6 kickoff + enumerate supported types</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Purpose: produce repeatable measured metrics — not estimates — for ingestion, extraction, embedding, memory, and search/chat latency.
-Steps: build parameterized harness under /benchmarks/; output machine-readable reports.</t>
+          <t>Purpose: list what content-core actually supports today and what needs work (OCR, EPUB, upload HTML, etc.).
+Steps: inventory from real code/config; note gaps; create wp-6-benchmarks. Can run after WP0; needs target hardware for later measurement tasks.</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>/benchmarks/ harness</t>
+          <t>Type inventory</t>
         </is>
       </c>
       <c r="F86" s="22" t="inlineStr">
@@ -7802,21 +7841,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G86" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G86" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="I86" s="17" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="J86" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K86" s="17" t="n"/>
       <c r="L86" s="18" t="n">
@@ -7828,24 +7867,28 @@
         </is>
       </c>
       <c r="N86" s="19" t="n">
+        <v>46266</v>
+      </c>
+      <c r="O86" s="19" t="n">
         <v>46267</v>
-      </c>
-      <c r="O86" s="19" t="n">
-        <v>46270</v>
       </c>
       <c r="P86" s="3" t="n"/>
       <c r="Q86" s="3" t="inlineStr">
         <is>
-          <t>Harness runs repeatably and outputs a metrics report</t>
-        </is>
-      </c>
-      <c r="R86" s="3" t="inlineStr"/>
+          <t>Supported types documented from real code</t>
+        </is>
+      </c>
+      <c r="R86" s="3" t="inlineStr">
+        <is>
+          <t>No guessed client-facing numbers</t>
+        </is>
+      </c>
       <c r="S86" s="3" t="inlineStr"/>
     </row>
     <row r="87" ht="75" customHeight="1">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -7855,18 +7898,18 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Assemble representative corpus</t>
+          <t>Build /benchmarks/ harness</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Purpose: find empirical slowdown/failure points across sizes and types.
-Steps: assemble small/medium/large/very-large docs plus scanned PDF, audio, and web page; ensure corpus licensing is clean for redistribution in-repo if needed.</t>
+          <t>Purpose: produce repeatable measured metrics — not estimates — for ingestion, extraction, embedding, memory, and search/chat latency.
+Steps: build parameterized harness under /benchmarks/; output machine-readable reports.</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>Fixed corpus under benchmarks/</t>
+          <t>/benchmarks/ harness</t>
         </is>
       </c>
       <c r="F87" s="22" t="inlineStr">
@@ -7881,14 +7924,14 @@
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="I87" s="17" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="J87" s="17" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="K87" s="17" t="n"/>
       <c r="L87" s="18" t="n">
@@ -7900,15 +7943,15 @@
         </is>
       </c>
       <c r="N87" s="19" t="n">
+        <v>46267</v>
+      </c>
+      <c r="O87" s="19" t="n">
         <v>46270</v>
-      </c>
-      <c r="O87" s="19" t="n">
-        <v>46273</v>
       </c>
       <c r="P87" s="3" t="n"/>
       <c r="Q87" s="3" t="inlineStr">
         <is>
-          <t>Corpus covers the size/type matrix</t>
+          <t>Harness runs repeatably and outputs a metrics report</t>
         </is>
       </c>
       <c r="R87" s="3" t="inlineStr"/>
@@ -7917,7 +7960,7 @@
     <row r="88" ht="75" customHeight="1">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
@@ -7927,18 +7970,18 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>Define accuracy methodology</t>
+          <t>Assemble representative corpus</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Purpose: define how accuracy is measured so client claims are defensible.
-Steps: specify extraction fidelity, retrieval relevance (labeled Q&amp;A), and chat groundedness methods; report per model tier.</t>
+          <t>Purpose: find empirical slowdown/failure points across sizes and types.
+Steps: assemble small/medium/large/very-large docs plus scanned PDF, audio, and web page; ensure corpus licensing is clean for redistribution in-repo if needed.</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>Accuracy method doc section</t>
+          <t>Fixed corpus under benchmarks/</t>
         </is>
       </c>
       <c r="F88" s="22" t="inlineStr">
@@ -7957,10 +8000,10 @@
         </is>
       </c>
       <c r="I88" s="17" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="J88" s="17" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="K88" s="17" t="n"/>
       <c r="L88" s="18" t="n">
@@ -7980,7 +8023,7 @@
       <c r="P88" s="3" t="n"/>
       <c r="Q88" s="3" t="inlineStr">
         <is>
-          <t>Accuracy reported as method + numbers</t>
+          <t>Corpus covers the size/type matrix</t>
         </is>
       </c>
       <c r="R88" s="3" t="inlineStr"/>
@@ -7989,7 +8032,7 @@
     <row r="89" ht="75" customHeight="1">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>8.3</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -7999,18 +8042,18 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>Run ≥2 hardware profiles</t>
+          <t>Define accuracy methodology</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Purpose: gather real numbers on bare-minimum and recommended hardware.
-Steps: run harness on both profiles; record figures; note local-model vs API-provider resource differences. Requires access to target hardware.</t>
+          <t>Purpose: define how accuracy is measured so client claims are defensible.
+Steps: specify extraction fidelity, retrieval relevance (labeled Q&amp;A), and chat groundedness methods; report per model tier.</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>Raw results JSON/CSV</t>
+          <t>Accuracy method doc section</t>
         </is>
       </c>
       <c r="F89" s="22" t="inlineStr">
@@ -8018,21 +8061,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G89" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G89" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>8.2,8.3</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="I89" s="17" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="J89" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K89" s="17" t="n"/>
       <c r="L89" s="18" t="n">
@@ -8044,28 +8087,24 @@
         </is>
       </c>
       <c r="N89" s="19" t="n">
+        <v>46270</v>
+      </c>
+      <c r="O89" s="19" t="n">
         <v>46273</v>
-      </c>
-      <c r="O89" s="19" t="n">
-        <v>46276</v>
       </c>
       <c r="P89" s="3" t="n"/>
       <c r="Q89" s="3" t="inlineStr">
         <is>
-          <t>Real measured numbers for both profiles</t>
-        </is>
-      </c>
-      <c r="R89" s="3" t="inlineStr">
-        <is>
-          <t>Hardware access is a dependency</t>
-        </is>
-      </c>
+          <t>Accuracy reported as method + numbers</t>
+        </is>
+      </c>
+      <c r="R89" s="3" t="inlineStr"/>
       <c r="S89" s="3" t="inlineStr"/>
     </row>
     <row r="90" ht="75" customHeight="1">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
@@ -8075,18 +8114,18 @@
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>docs/PERFORMANCE_AND_SIZING.md + review</t>
+          <t>Run ≥2 hardware profiles</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Purpose: publish client-facing sizing guidance backed only by harness output.
-Steps: write types, limits, times, accuracy, min vs recommended hardware; peer review; merge.</t>
+          <t>Purpose: gather real numbers on bare-minimum and recommended hardware.
+Steps: run harness on both profiles; record figures; note local-model vs API-provider resource differences. Requires access to target hardware.</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>docs/PERFORMANCE_AND_SIZING.md</t>
+          <t>Raw results JSON/CSV</t>
         </is>
       </c>
       <c r="F90" s="22" t="inlineStr">
@@ -8094,21 +8133,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G90" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G90" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>8.2,8.3</t>
         </is>
       </c>
       <c r="I90" s="17" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="J90" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K90" s="17" t="n"/>
       <c r="L90" s="18" t="n">
@@ -8120,45 +8159,49 @@
         </is>
       </c>
       <c r="N90" s="19" t="n">
+        <v>46273</v>
+      </c>
+      <c r="O90" s="19" t="n">
         <v>46276</v>
-      </c>
-      <c r="O90" s="19" t="n">
-        <v>46277</v>
       </c>
       <c r="P90" s="3" t="n"/>
       <c r="Q90" s="3" t="inlineStr">
         <is>
-          <t>Doc contains measured numbers only</t>
-        </is>
-      </c>
-      <c r="R90" s="3" t="inlineStr"/>
+          <t>Real measured numbers for both profiles</t>
+        </is>
+      </c>
+      <c r="R90" s="3" t="inlineStr">
+        <is>
+          <t>Hardware access is a dependency</t>
+        </is>
+      </c>
       <c r="S90" s="3" t="inlineStr"/>
     </row>
     <row r="91" ht="75" customHeight="1">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>WP7 — Cross-platform Packaging</t>
+          <t>WP6 — Doc Processing Benchmarks</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>WP7 kickoff</t>
+          <t>docs/PERFORMANCE_AND_SIZING.md + review</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Purpose: package the real authenticated + branded app, not the pre-WP2 password prototype.
-Steps: create wp-7-packaging only after WP2 and WP3 are on main.</t>
+          <t>Purpose: publish client-facing sizing guidance backed only by harness output.
+Steps: write types, limits, times, accuracy, min vs recommended hardware; peer review; merge.</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>Branch</t>
+          <t>docs/PERFORMANCE_AND_SIZING.md</t>
         </is>
       </c>
       <c r="F91" s="22" t="inlineStr">
@@ -8173,14 +8216,14 @@
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>5.6,4.10</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="I91" s="17" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J91" s="17" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="K91" s="17" t="n"/>
       <c r="L91" s="18" t="n">
@@ -8192,15 +8235,15 @@
         </is>
       </c>
       <c r="N91" s="19" t="n">
-        <v>46283</v>
+        <v>46276</v>
       </c>
       <c r="O91" s="19" t="n">
-        <v>46283</v>
+        <v>46277</v>
       </c>
       <c r="P91" s="3" t="n"/>
       <c r="Q91" s="3" t="inlineStr">
         <is>
-          <t>Starts only after branded + authenticated app exists</t>
+          <t>Doc contains measured numbers only</t>
         </is>
       </c>
       <c r="R91" s="3" t="inlineStr"/>
@@ -8209,7 +8252,7 @@
     <row r="92" ht="75" customHeight="1">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -8219,18 +8262,18 @@
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Verify Docker Compose on Windows + Linux</t>
+          <t>WP7 kickoff</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Purpose: make containers the recommended identical path on both OSes.
-Steps: verify docker-compose and Dockerfile.single on Docker Desktop/WSL2 and Linux; document as primary deploy path.</t>
+          <t>Purpose: package the real authenticated + branded app, not the pre-WP2 password prototype.
+Steps: create wp-7-packaging only after WP2 and WP3 are on main.</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>Verified container deploy</t>
+          <t>Branch</t>
         </is>
       </c>
       <c r="F92" s="22" t="inlineStr">
@@ -8238,21 +8281,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G92" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G92" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>5.6,4.10</t>
         </is>
       </c>
       <c r="I92" s="17" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="J92" s="17" t="n">
-        <v>2</v>
+        <v>0.25</v>
       </c>
       <c r="K92" s="17" t="n"/>
       <c r="L92" s="18" t="n">
@@ -8260,19 +8303,19 @@
       </c>
       <c r="M92" s="3" t="inlineStr">
         <is>
-          <t>DevOps / Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N92" s="19" t="n">
         <v>46283</v>
       </c>
       <c r="O92" s="19" t="n">
-        <v>46287</v>
+        <v>46283</v>
       </c>
       <c r="P92" s="3" t="n"/>
       <c r="Q92" s="3" t="inlineStr">
         <is>
-          <t>Container deployment verified on both OSes</t>
+          <t>Starts only after branded + authenticated app exists</t>
         </is>
       </c>
       <c r="R92" s="3" t="inlineStr"/>
@@ -8281,7 +8324,7 @@
     <row r="93" ht="75" customHeight="1">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -8291,18 +8334,18 @@
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>Native Linux install path (systemd)</t>
+          <t>Verify Docker Compose on Windows + Linux</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>Purpose: support customers who refuse containers.
-Steps: systemd units + install script; document dependencies for common distros; verify on at least one distro.</t>
+          <t>Purpose: make containers the recommended identical path on both OSes.
+Steps: verify docker-compose and Dockerfile.single on Docker Desktop/WSL2 and Linux; document as primary deploy path.</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>Linux native docs + scripts</t>
+          <t>Verified container deploy</t>
         </is>
       </c>
       <c r="F93" s="22" t="inlineStr">
@@ -8310,14 +8353,14 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G93" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G93" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="I93" s="17" t="n">
@@ -8336,15 +8379,15 @@
         </is>
       </c>
       <c r="N93" s="19" t="n">
+        <v>46283</v>
+      </c>
+      <c r="O93" s="19" t="n">
         <v>46287</v>
-      </c>
-      <c r="O93" s="19" t="n">
-        <v>46289</v>
       </c>
       <c r="P93" s="3" t="n"/>
       <c r="Q93" s="3" t="inlineStr">
         <is>
-          <t>Verified on ≥1 Linux distro</t>
+          <t>Container deployment verified on both OSes</t>
         </is>
       </c>
       <c r="R93" s="3" t="inlineStr"/>
@@ -8353,7 +8396,7 @@
     <row r="94" ht="75" customHeight="1">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>9.3</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -8363,18 +8406,18 @@
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>Native Windows Service path</t>
+          <t>Native Linux install path (systemd)</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Purpose: support Windows Server native installs.
-Steps: Windows Service wrapper; SurrealDB-on-Windows notes; frontend serve docs; verify on Windows Server or equivalent.</t>
+          <t>Purpose: support customers who refuse containers.
+Steps: systemd units + install script; document dependencies for common distros; verify on at least one distro.</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Windows native docs + scripts</t>
+          <t>Linux native docs + scripts</t>
         </is>
       </c>
       <c r="F94" s="22" t="inlineStr">
@@ -8416,7 +8459,7 @@
       <c r="P94" s="3" t="n"/>
       <c r="Q94" s="3" t="inlineStr">
         <is>
-          <t>Verified on Windows Server or equivalent</t>
+          <t>Verified on ≥1 Linux distro</t>
         </is>
       </c>
       <c r="R94" s="3" t="inlineStr"/>
@@ -8425,7 +8468,7 @@
     <row r="95" ht="75" customHeight="1">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>9.4</t>
+          <t>9.3</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -8435,18 +8478,18 @@
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>Installer helper CLI (interactive + non-interactive)</t>
+          <t>Native Windows Service path</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>Purpose: let a non-expert stand up a branded client instance without hand-editing half a dozen files.
-Steps: CLI for prereq check → collect brand/Entra/provider/DB/encryption → write config → migrate → start → health check; add scripted/non-interactive mode for repeatable installs.</t>
+          <t>Purpose: support Windows Server native installs.
+Steps: Windows Service wrapper; SurrealDB-on-Windows notes; frontend serve docs; verify on Windows Server or equivalent.</t>
         </is>
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>onboard/install CLI</t>
+          <t>Windows native docs + scripts</t>
         </is>
       </c>
       <c r="F95" s="22" t="inlineStr">
@@ -8454,21 +8497,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G95" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G95" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>9.1,5.4</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="I95" s="17" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="J95" s="17" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K95" s="17" t="n"/>
       <c r="L95" s="18" t="n">
@@ -8476,32 +8519,28 @@
       </c>
       <c r="M95" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>DevOps / Engineer</t>
         </is>
       </c>
       <c r="N95" s="19" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O95" s="19" t="n">
         <v>46289</v>
-      </c>
-      <c r="O95" s="19" t="n">
-        <v>46295</v>
       </c>
       <c r="P95" s="3" t="n"/>
       <c r="Q95" s="3" t="inlineStr">
         <is>
-          <t>Full install in both modes; scripted branded client stand-up works</t>
-        </is>
-      </c>
-      <c r="R95" s="3" t="inlineStr">
-        <is>
-          <t>Deployment counterpart to WP3 theming</t>
-        </is>
-      </c>
+          <t>Verified on Windows Server or equivalent</t>
+        </is>
+      </c>
+      <c r="R95" s="3" t="inlineStr"/>
       <c r="S95" s="3" t="inlineStr"/>
     </row>
     <row r="96" ht="75" customHeight="1">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>9.4</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
@@ -8511,18 +8550,18 @@
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>docs/DEPLOYMENT.md + WP7 review</t>
+          <t>Installer helper CLI (interactive + non-interactive)</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Purpose: one operator guide for container + native + CLI paths.
-Steps: write DEPLOYMENT.md; verify WP7 ACs; PR; human review.</t>
+          <t>Purpose: let a non-expert stand up a branded client instance without hand-editing half a dozen files.
+Steps: CLI for prereq check → collect brand/Entra/provider/DB/encryption → write config → migrate → start → health check; add scripted/non-interactive mode for repeatable installs.</t>
         </is>
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>docs/DEPLOYMENT.md</t>
+          <t>onboard/install CLI</t>
         </is>
       </c>
       <c r="F96" s="22" t="inlineStr">
@@ -8530,21 +8569,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G96" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G96" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>9.2,9.3,9.4</t>
+          <t>9.1,5.4</t>
         </is>
       </c>
       <c r="I96" s="17" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="J96" s="17" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K96" s="17" t="n"/>
       <c r="L96" s="18" t="n">
@@ -8552,49 +8591,53 @@
       </c>
       <c r="M96" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N96" s="19" t="n">
+        <v>46289</v>
+      </c>
+      <c r="O96" s="19" t="n">
         <v>46295</v>
-      </c>
-      <c r="O96" s="19" t="n">
-        <v>46296</v>
       </c>
       <c r="P96" s="3" t="n"/>
       <c r="Q96" s="3" t="inlineStr">
         <is>
-          <t>All WP7 acceptance criteria pass</t>
-        </is>
-      </c>
-      <c r="R96" s="3" t="inlineStr"/>
+          <t>Full install in both modes; scripted branded client stand-up works</t>
+        </is>
+      </c>
+      <c r="R96" s="3" t="inlineStr">
+        <is>
+          <t>Deployment counterpart to WP3 theming</t>
+        </is>
+      </c>
       <c r="S96" s="3" t="inlineStr"/>
     </row>
     <row r="97" ht="75" customHeight="1">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>WP8 — Onboarding &amp; In-app Help</t>
+          <t>WP7 — Cross-platform Packaging</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>WP8 kickoff (LAST)</t>
+          <t>docs/DEPLOYMENT.md + WP7 review</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>Purpose: build onboarding against final flows only — wizard/tour copy must match the shipped product.
-Steps: create wp-8-onboarding after WP2/3/5/7 are stable on main.</t>
+          <t>Purpose: one operator guide for container + native + CLI paths.
+Steps: write DEPLOYMENT.md; verify WP7 ACs; PR; human review.</t>
         </is>
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>Branch</t>
+          <t>docs/DEPLOYMENT.md</t>
         </is>
       </c>
       <c r="F97" s="22" t="inlineStr">
@@ -8602,21 +8645,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G97" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G97" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
-          <t>9.5,7.6,5.6</t>
+          <t>9.2,9.3,9.4</t>
         </is>
       </c>
       <c r="I97" s="17" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J97" s="17" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="K97" s="17" t="n"/>
       <c r="L97" s="18" t="n">
@@ -8624,32 +8667,28 @@
       </c>
       <c r="M97" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N97" s="19" t="n">
-        <v>46297</v>
+        <v>46295</v>
       </c>
       <c r="O97" s="19" t="n">
-        <v>46297</v>
+        <v>46296</v>
       </c>
       <c r="P97" s="3" t="n"/>
       <c r="Q97" s="3" t="inlineStr">
         <is>
-          <t>Built against final UX</t>
-        </is>
-      </c>
-      <c r="R97" s="3" t="inlineStr">
-        <is>
-          <t>Must be last in the program sequence</t>
-        </is>
-      </c>
+          <t>All WP7 acceptance criteria pass</t>
+        </is>
+      </c>
+      <c r="R97" s="3" t="inlineStr"/>
       <c r="S97" s="3" t="inlineStr"/>
     </row>
     <row r="98" ht="75" customHeight="1">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
@@ -8659,18 +8698,18 @@
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>First-run / admin setup wizard</t>
+          <t>WP8 kickoff (LAST)</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>Purpose: take a fresh instance to a working configured app without tribal knowledge.
-Steps: detect fresh instance; guide providers/keys, models, brand (admin), connect a source, create first notebook; all copy via i18n.</t>
+          <t>Purpose: build onboarding against final flows only — wizard/tour copy must match the shipped product.
+Steps: create wp-8-onboarding after WP2/3/5/7 are stable on main.</t>
         </is>
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>Setup wizard</t>
+          <t>Branch</t>
         </is>
       </c>
       <c r="F98" s="22" t="inlineStr">
@@ -8678,21 +8717,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G98" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G98" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>9.5,7.6,5.6</t>
         </is>
       </c>
       <c r="I98" s="17" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="J98" s="17" t="n">
-        <v>3</v>
+        <v>0.25</v>
       </c>
       <c r="K98" s="17" t="n"/>
       <c r="L98" s="18" t="n">
@@ -8707,21 +8746,25 @@
         <v>46297</v>
       </c>
       <c r="O98" s="19" t="n">
-        <v>46302</v>
+        <v>46297</v>
       </c>
       <c r="P98" s="3" t="n"/>
       <c r="Q98" s="3" t="inlineStr">
         <is>
-          <t>Completing the wizard leaves a working configured app</t>
-        </is>
-      </c>
-      <c r="R98" s="3" t="inlineStr"/>
+          <t>Built against final UX</t>
+        </is>
+      </c>
+      <c r="R98" s="3" t="inlineStr">
+        <is>
+          <t>Must be last in the program sequence</t>
+        </is>
+      </c>
       <c r="S98" s="3" t="inlineStr"/>
     </row>
     <row r="99" ht="75" customHeight="1">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
@@ -8731,18 +8774,18 @@
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>User guided tour (core loop)</t>
+          <t>First-run / admin setup wizard</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>Purpose: teach the core loop — add source → search → chat → transform → podcast — with an accessible spotlight tour.
-Steps: implement dismissible/resumable tour; keep steps short; i18n all locales.</t>
+          <t>Purpose: take a fresh instance to a working configured app without tribal knowledge.
+Steps: detect fresh instance; guide providers/keys, models, brand (admin), connect a source, create first notebook; all copy via i18n.</t>
         </is>
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>Guided tour</t>
+          <t>Setup wizard</t>
         </is>
       </c>
       <c r="F99" s="22" t="inlineStr">
@@ -8757,14 +8800,14 @@
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="I99" s="17" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="J99" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K99" s="17" t="n"/>
       <c r="L99" s="18" t="n">
@@ -8776,15 +8819,15 @@
         </is>
       </c>
       <c r="N99" s="19" t="n">
+        <v>46297</v>
+      </c>
+      <c r="O99" s="19" t="n">
         <v>46302</v>
-      </c>
-      <c r="O99" s="19" t="n">
-        <v>46304</v>
       </c>
       <c r="P99" s="3" t="n"/>
       <c r="Q99" s="3" t="inlineStr">
         <is>
-          <t>New user can complete the core-loop tour</t>
+          <t>Completing the wizard leaves a working configured app</t>
         </is>
       </c>
       <c r="R99" s="3" t="inlineStr"/>
@@ -8793,7 +8836,7 @@
     <row r="100" ht="75" customHeight="1">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
@@ -8803,18 +8846,18 @@
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>Contextual tooltips + empty states + help surface</t>
+          <t>User guided tour (core loop)</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>Purpose: remove dead-ends for new users on every main screen.
-Steps: tooltips on non-obvious controls; useful empty states; persistent help (docs, shortcuts, restart tour, BrandConfig support URL); all strings in i18n.</t>
+          <t>Purpose: teach the core loop — add source → search → chat → transform → podcast — with an accessible spotlight tour.
+Steps: implement dismissible/resumable tour; keep steps short; i18n all locales.</t>
         </is>
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>Tooltips/empty states/help</t>
+          <t>Guided tour</t>
         </is>
       </c>
       <c r="F100" s="22" t="inlineStr">
@@ -8822,21 +8865,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G100" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G100" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="I100" s="17" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J100" s="17" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="K100" s="17" t="n"/>
       <c r="L100" s="18" t="n">
@@ -8848,28 +8891,24 @@
         </is>
       </c>
       <c r="N100" s="19" t="n">
+        <v>46302</v>
+      </c>
+      <c r="O100" s="19" t="n">
         <v>46304</v>
-      </c>
-      <c r="O100" s="19" t="n">
-        <v>46309</v>
       </c>
       <c r="P100" s="3" t="n"/>
       <c r="Q100" s="3" t="inlineStr">
         <is>
-          <t>All copy in i18n; help reachable everywhere</t>
-        </is>
-      </c>
-      <c r="R100" s="3" t="inlineStr">
-        <is>
-          <t>Locale parity required across all locales</t>
-        </is>
-      </c>
+          <t>New user can complete the core-loop tour</t>
+        </is>
+      </c>
+      <c r="R100" s="3" t="inlineStr"/>
       <c r="S100" s="3" t="inlineStr"/>
     </row>
     <row r="101" ht="75" customHeight="1">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>10.3</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -8879,18 +8918,18 @@
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>docs/ONBOARDING.md + program close review</t>
+          <t>Contextual tooltips + empty states + help surface</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>Purpose: document onboarding structure and verify program-level definition of done.
-Steps: write ONBOARDING.md; confirm a new client can be stood up by config + installer only (branded, Entra-auth’d, connectors, Windows/Linux) without per-client code rebuilds.</t>
+          <t>Purpose: remove dead-ends for new users on every main screen.
+Steps: tooltips on non-obvious controls; useful empty states; persistent help (docs, shortcuts, restart tour, BrandConfig support URL); all strings in i18n.</t>
         </is>
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>docs/ONBOARDING.md; program DoD check</t>
+          <t>Tooltips/empty states/help</t>
         </is>
       </c>
       <c r="F101" s="22" t="inlineStr">
@@ -8905,14 +8944,14 @@
       </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="I101" s="17" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="J101" s="17" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="K101" s="17" t="n"/>
       <c r="L101" s="18" t="n">
@@ -8920,26 +8959,102 @@
       </c>
       <c r="M101" s="3" t="inlineStr">
         <is>
-          <t>Engineering Lead</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N101" s="19" t="n">
+        <v>46304</v>
+      </c>
+      <c r="O101" s="19" t="n">
         <v>46309</v>
-      </c>
-      <c r="O101" s="19" t="n">
-        <v>46310</v>
       </c>
       <c r="P101" s="3" t="n"/>
       <c r="Q101" s="3" t="inlineStr">
         <is>
+          <t>All copy in i18n; help reachable everywhere</t>
+        </is>
+      </c>
+      <c r="R101" s="3" t="inlineStr">
+        <is>
+          <t>Locale parity required across all locales</t>
+        </is>
+      </c>
+      <c r="S101" s="3" t="inlineStr"/>
+    </row>
+    <row r="102" ht="75" customHeight="1">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>10.4</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>WP8 — Onboarding &amp; In-app Help</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>docs/ONBOARDING.md + program close review</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: document onboarding structure and verify program-level definition of done.
+Steps: write ONBOARDING.md; confirm a new client can be stood up by config + installer only (branded, Entra-auth’d, connectors, Windows/Linux) without per-client code rebuilds.</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>docs/ONBOARDING.md; program DoD check</t>
+        </is>
+      </c>
+      <c r="F102" s="22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G102" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H102" s="3" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="I102" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="J102" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K102" s="17" t="n"/>
+      <c r="L102" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M102" s="3" t="inlineStr">
+        <is>
+          <t>Engineering Lead</t>
+        </is>
+      </c>
+      <c r="N102" s="19" t="n">
+        <v>46309</v>
+      </c>
+      <c r="O102" s="19" t="n">
+        <v>46310</v>
+      </c>
+      <c r="P102" s="3" t="n"/>
+      <c r="Q102" s="3" t="inlineStr">
+        <is>
           <t>All WP8 ACs + program definition of done satisfied</t>
         </is>
       </c>
-      <c r="R101" s="3" t="inlineStr"/>
-      <c r="S101" s="3" t="inlineStr"/>
+      <c r="R102" s="3" t="inlineStr"/>
+      <c r="S102" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A5:S101"/>
+  <autoFilter ref="A5:S102"/>
   <mergeCells count="3">
     <mergeCell ref="A3:S3"/>
     <mergeCell ref="A2:S2"/>
@@ -9010,7 +9125,7 @@
           <t>Clean build reproducible from docs/DEV_SETUP.md</t>
         </is>
       </c>
-      <c r="C4" s="26" t="inlineStr">
+      <c r="C4" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9033,7 +9148,7 @@
           <t>upstream-base tag exists; upstream remote configured</t>
         </is>
       </c>
-      <c r="C5" s="26" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9060,7 +9175,7 @@
           <t>Characterization tests: ingestion, search, chat, notebook CRUD</t>
         </is>
       </c>
-      <c r="C6" s="26" t="inlineStr">
+      <c r="C6" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9083,7 +9198,7 @@
           <t>CI runs on PR and blocks merge on failure</t>
         </is>
       </c>
-      <c r="C7" s="26" t="inlineStr">
+      <c r="C7" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9106,7 +9221,7 @@
           <t>License scan runs in CI and passes</t>
         </is>
       </c>
-      <c r="C8" s="26" t="inlineStr">
+      <c r="C8" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9129,7 +9244,7 @@
           <t>LICENSE retains upstream copyright + our copyright</t>
         </is>
       </c>
-      <c r="C9" s="26" t="inlineStr">
+      <c r="C9" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9156,7 +9271,7 @@
           <t>THIRD-PARTY-NOTICES.md complete and reproducible</t>
         </is>
       </c>
-      <c r="C10" s="26" t="inlineStr">
+      <c r="C10" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9183,7 +9298,7 @@
           <t>SurrealDB BSL entry present and accurate</t>
         </is>
       </c>
-      <c r="C11" s="26" t="inlineStr">
+      <c r="C11" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9206,7 +9321,7 @@
           <t>pycountry unmodified; CI asserts</t>
         </is>
       </c>
-      <c r="C12" s="26" t="inlineStr">
+      <c r="C12" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9229,7 +9344,7 @@
           <t>docs/PROVIDER_TERMS.md exists</t>
         </is>
       </c>
-      <c r="C13" s="26" t="inlineStr">
+      <c r="C13" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9256,7 +9371,7 @@
           <t>No secrets committed; encryption key handling documented</t>
         </is>
       </c>
-      <c r="C14" s="26" t="inlineStr">
+      <c r="C14" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9279,7 +9394,7 @@
           <t>Tenancy model chosen and documented</t>
         </is>
       </c>
-      <c r="C15" s="26" t="inlineStr">
+      <c r="C15" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9306,7 +9421,7 @@
           <t>Login via real Entra account E2E</t>
         </is>
       </c>
-      <c r="C16" s="27" t="inlineStr">
+      <c r="C16" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9329,7 +9444,7 @@
           <t>Every API request validates Entra JWT (iss/aud/sig/exp)</t>
         </is>
       </c>
-      <c r="C17" s="27" t="inlineStr">
+      <c r="C17" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9348,7 +9463,7 @@
           <t>Users JIT-provisioned; user record after first login</t>
         </is>
       </c>
-      <c r="C18" s="27" t="inlineStr">
+      <c r="C18" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9367,7 +9482,7 @@
           <t>Roles enforced on sensitive routes (403)</t>
         </is>
       </c>
-      <c r="C19" s="27" t="inlineStr">
+      <c r="C19" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9386,7 +9501,7 @@
           <t>Users only see own notebooks/sources</t>
         </is>
       </c>
-      <c r="C20" s="27" t="inlineStr">
+      <c r="C20" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9405,7 +9520,7 @@
           <t>Password provider still works as local-dev fallback</t>
         </is>
       </c>
-      <c r="C21" s="27" t="inlineStr">
+      <c r="C21" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9424,7 +9539,7 @@
           <t>Second provider needs no route-handler changes (stub)</t>
         </is>
       </c>
-      <c r="C22" s="27" t="inlineStr">
+      <c r="C22" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9443,7 +9558,7 @@
           <t>docs/AUTH.md complete</t>
         </is>
       </c>
-      <c r="C23" s="27" t="inlineStr">
+      <c r="C23" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9462,7 +9577,7 @@
           <t>FRONTEND_MAP.md complete with where-to-change table</t>
         </is>
       </c>
-      <c r="C24" s="27" t="inlineStr">
+      <c r="C24" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9481,7 +9596,7 @@
           <t>New client branded by config only (two brands, same build)</t>
         </is>
       </c>
-      <c r="C25" s="27" t="inlineStr">
+      <c r="C25" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9500,7 +9615,7 @@
           <t>Hardcoded brand strings/assets read from BrandConfig</t>
         </is>
       </c>
-      <c r="C26" s="27" t="inlineStr">
+      <c r="C26" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9519,7 +9634,7 @@
           <t>Dark/light both themed correctly</t>
         </is>
       </c>
-      <c r="C27" s="27" t="inlineStr">
+      <c r="C27" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9538,13 +9653,21 @@
           <t>Every router/endpoint documented with auth + models</t>
         </is>
       </c>
-      <c r="C28" s="27" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr"/>
-      <c r="E28" s="3" t="inlineStr"/>
+      <c r="C28" s="25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>docs/BACKEND_MAP.md</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>PR #55</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -9557,13 +9680,21 @@
           <t>Every domain model and graph documented</t>
         </is>
       </c>
-      <c r="C29" s="27" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
+      <c r="C29" s="25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>docs/BACKEND_MAP.md</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>PR #55</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -9576,13 +9707,21 @@
           <t>Five how-to-add-X playbooks present</t>
         </is>
       </c>
-      <c r="C30" s="27" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr"/>
-      <c r="E30" s="3" t="inlineStr"/>
+      <c r="C30" s="25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>docs/BACKEND_MAP.md</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>PR #55</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -9595,13 +9734,21 @@
           <t>New engineer can locate changes using only BACKEND_MAP</t>
         </is>
       </c>
-      <c r="C31" s="27" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
+      <c r="C31" s="25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>docs/BACKEND_MAP.md</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>tests/test_backend_map.py</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -9614,7 +9761,7 @@
           <t>SharePoint connect → folder → pull all supported docs</t>
         </is>
       </c>
-      <c r="C32" s="27" t="inlineStr">
+      <c r="C32" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9633,7 +9780,7 @@
           <t>Ingestion reuses existing pipeline</t>
         </is>
       </c>
-      <c r="C33" s="27" t="inlineStr">
+      <c r="C33" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9652,7 +9799,7 @@
           <t>Batch per-doc progress; single failure non-fatal</t>
         </is>
       </c>
-      <c r="C34" s="27" t="inlineStr">
+      <c r="C34" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9671,7 +9818,7 @@
           <t>Chat across whole pulled set</t>
         </is>
       </c>
-      <c r="C35" s="27" t="inlineStr">
+      <c r="C35" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9690,7 +9837,7 @@
           <t>Tokens encrypted per user; source permissions respected</t>
         </is>
       </c>
-      <c r="C36" s="27" t="inlineStr">
+      <c r="C36" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9709,7 +9856,7 @@
           <t>New connector = SourceConnector interface only</t>
         </is>
       </c>
-      <c r="C37" s="27" t="inlineStr">
+      <c r="C37" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9728,7 +9875,7 @@
           <t>docs/CONNECTORS.md complete</t>
         </is>
       </c>
-      <c r="C38" s="27" t="inlineStr">
+      <c r="C38" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9747,7 +9894,7 @@
           <t>Benchmark harness repeatable with metrics report</t>
         </is>
       </c>
-      <c r="C39" s="27" t="inlineStr">
+      <c r="C39" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9766,7 +9913,7 @@
           <t>PERFORMANCE_AND_SIZING.md has measured numbers (2 profiles)</t>
         </is>
       </c>
-      <c r="C40" s="27" t="inlineStr">
+      <c r="C40" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9785,7 +9932,7 @@
           <t>Supported types + tested size limits + failure points</t>
         </is>
       </c>
-      <c r="C41" s="27" t="inlineStr">
+      <c r="C41" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9804,7 +9951,7 @@
           <t>Accuracy methodology + results per model tier</t>
         </is>
       </c>
-      <c r="C42" s="27" t="inlineStr">
+      <c r="C42" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9823,7 +9970,7 @@
           <t>Min vs recommended hardware justified by numbers</t>
         </is>
       </c>
-      <c r="C43" s="27" t="inlineStr">
+      <c r="C43" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9842,7 +9989,7 @@
           <t>Container deploy verified Windows + Linux</t>
         </is>
       </c>
-      <c r="C44" s="27" t="inlineStr">
+      <c r="C44" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9861,7 +10008,7 @@
           <t>Native install documented/verified Linux + Windows</t>
         </is>
       </c>
-      <c r="C45" s="27" t="inlineStr">
+      <c r="C45" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9880,7 +10027,7 @@
           <t>Installer CLI full install interactive + non-interactive</t>
         </is>
       </c>
-      <c r="C46" s="27" t="inlineStr">
+      <c r="C46" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9899,7 +10046,7 @@
           <t>Scripted install stands up branded client E2E</t>
         </is>
       </c>
-      <c r="C47" s="27" t="inlineStr">
+      <c r="C47" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9918,7 +10065,7 @@
           <t>docs/DEPLOYMENT.md complete</t>
         </is>
       </c>
-      <c r="C48" s="27" t="inlineStr">
+      <c r="C48" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9937,7 +10084,7 @@
           <t>Fresh instance launches setup wizard → working app</t>
         </is>
       </c>
-      <c r="C49" s="27" t="inlineStr">
+      <c r="C49" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9956,7 +10103,7 @@
           <t>Guided tour of core loop completable</t>
         </is>
       </c>
-      <c r="C50" s="27" t="inlineStr">
+      <c r="C50" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9975,7 +10122,7 @@
           <t>Contextual tooltips; all copy in i18n</t>
         </is>
       </c>
-      <c r="C51" s="27" t="inlineStr">
+      <c r="C51" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9994,7 +10141,7 @@
           <t>Every main screen useful empty state</t>
         </is>
       </c>
-      <c r="C52" s="27" t="inlineStr">
+      <c r="C52" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -10013,7 +10160,7 @@
           <t>Tour dismissible/resumable; help surface everywhere</t>
         </is>
       </c>
-      <c r="C53" s="27" t="inlineStr">
+      <c r="C53" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -10032,7 +10179,7 @@
           <t>docs/ONBOARDING.md complete</t>
         </is>
       </c>
-      <c r="C54" s="27" t="inlineStr">
+      <c r="C54" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -10051,7 +10198,7 @@
           <t>New client by config + installer only (no per-client rebuild)</t>
         </is>
       </c>
-      <c r="C55" s="27" t="inlineStr">
+      <c r="C55" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -10074,7 +10221,7 @@
           <t>Licensing compliant and drift-guarded</t>
         </is>
       </c>
-      <c r="C56" s="26" t="inlineStr">
+      <c r="C56" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -10097,7 +10244,7 @@
           <t>Real performance/sizing numbers for clients</t>
         </is>
       </c>
-      <c r="C57" s="27" t="inlineStr">
+      <c r="C57" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -10120,17 +10267,21 @@
           <t>Backend + frontend fully mapped</t>
         </is>
       </c>
-      <c r="C58" s="27" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C58" s="25" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>WP3a + WP4</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="inlineStr"/>
+          <t>docs/FRONTEND_MAP.md + docs/BACKEND_MAP.md</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>PR #55</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -10161,12 +10312,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="inlineStr">
+      <c r="A3" s="27" t="inlineStr">
         <is>
           <t>Topic</t>
         </is>
       </c>
-      <c r="B3" s="28" t="inlineStr">
+      <c r="B3" s="27" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>

</xml_diff>

<commit_message>
docs: mark WP4 done and ignore local docx files (#56)
* docs: mark WP4 done on the WBS.

Tasks 6.0-6.4 and the four backend-map acceptance rows now match PR #55.

Co-authored-by: Cursor <cursoragent@cursor.com>

* chore: keep local docx files out of git and images.

Co-authored-by: Cursor <cursoragent@cursor.com>

---------

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/commercialization/Open-Notebook-Commercialization-WBS-Task-Schedule.xlsx
+++ b/docs/commercialization/Open-Notebook-Commercialization-WBS-Task-Schedule.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estimating Assumptions" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'WBS Task List'!$A$5:$S$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'WBS Task List'!$A$5:$S$102</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -59,7 +59,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -94,11 +94,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E0E7FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
     <fill>
@@ -138,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -151,7 +146,7 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -192,13 +187,10 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -760,13 +752,13 @@
         <v>32</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>4</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.3125</v>
+        <v>0.375</v>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
@@ -871,7 +863,7 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>56</v>
+        <v>96</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
@@ -879,7 +871,7 @@
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>0</v>
@@ -931,16 +923,14 @@
       <c r="C14" s="3" t="n">
         <v>49</v>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D14" s="3" t="n">
+        <v>49</v>
       </c>
       <c r="E14" s="3" t="n">
         <v>6.2</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
@@ -1079,13 +1069,13 @@
         </is>
       </c>
       <c r="C20" s="8" t="n">
-        <v>1035</v>
+        <v>1075</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>439</v>
+        <v>489</v>
       </c>
       <c r="F20" s="9" t="n">
-        <v>0.4229951690821256</v>
+        <v>0.4546976744186046</v>
       </c>
     </row>
     <row r="22">
@@ -1102,7 +1092,7 @@
         </is>
       </c>
       <c r="B23" s="11" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="24">
@@ -1112,7 +1102,7 @@
         </is>
       </c>
       <c r="B24" s="11" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25">
@@ -1132,7 +1122,7 @@
         </is>
       </c>
       <c r="B26" s="11" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27">
@@ -1142,7 +1132,7 @@
         </is>
       </c>
       <c r="B27" s="11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1152,7 +1142,7 @@
         </is>
       </c>
       <c r="B28" s="11" t="n">
-        <v>597.2</v>
+        <v>586.2</v>
       </c>
     </row>
     <row r="29">
@@ -1162,7 +1152,7 @@
         </is>
       </c>
       <c r="B29" s="11" t="n">
-        <v>74.90000000000001</v>
+        <v>73.40000000000001</v>
       </c>
     </row>
     <row r="30">
@@ -1232,7 +1222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S101"/>
+  <dimension ref="A1:S102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4126,12 +4116,12 @@
           <t>Cleaner image; allowlist reduced</t>
         </is>
       </c>
-      <c r="F39" s="23" t="inlineStr">
-        <is>
-          <t>Blocked</t>
-        </is>
-      </c>
-      <c r="G39" s="24" t="inlineStr">
+      <c r="F39" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G39" s="23" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -4147,18 +4137,26 @@
       <c r="J39" s="17" t="n">
         <v>0.25</v>
       </c>
-      <c r="K39" s="17" t="n"/>
+      <c r="K39" s="17" t="n">
+        <v>1</v>
+      </c>
       <c r="L39" s="18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M39" s="3" t="inlineStr">
         <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="N39" s="3" t="n"/>
-      <c r="O39" s="3" t="n"/>
-      <c r="P39" s="3" t="n"/>
+      <c r="N39" s="19" t="n">
+        <v>46282</v>
+      </c>
+      <c r="O39" s="19" t="n">
+        <v>46282</v>
+      </c>
+      <c r="P39" s="19" t="n">
+        <v>46282</v>
+      </c>
       <c r="Q39" s="3" t="inlineStr">
         <is>
           <t>asciidoc gone from allowlist and Dockerfile</t>
@@ -4166,12 +4164,12 @@
       </c>
       <c r="R39" s="3" t="inlineStr">
         <is>
-          <t>Blocked on upstream PR</t>
+          <t>Upstream content-core#58 merged 2026-09-05 (v2.1.0); bumped and stripped in this fork</t>
         </is>
       </c>
       <c r="S39" s="3" t="inlineStr">
         <is>
-          <t>content-core#58</t>
+          <t>PR #23; content-core#58; content-core v2.1.0</t>
         </is>
       </c>
     </row>
@@ -6017,7 +6015,7 @@
           <t>docs/SHARING.md; branch ready for PR</t>
         </is>
       </c>
-      <c r="F62" s="25" t="inlineStr">
+      <c r="F62" s="24" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
@@ -6101,9 +6099,9 @@
           <t>Entra-backed groups with live membership</t>
         </is>
       </c>
-      <c r="F63" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="F63" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G63" s="16" t="inlineStr">
@@ -6146,7 +6144,7 @@
       </c>
       <c r="S63" s="3" t="inlineStr">
         <is>
-          <t>user_group.source / entra_group_oid; docs/SHARING.md</t>
+          <t>user_group.source / entra_group_oid; docs/SHARING.md; api/graph_client.py; commands/entra_group_sync.py</t>
         </is>
       </c>
     </row>
@@ -6163,24 +6161,24 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Full org directory user picker (Graph)</t>
+          <t>Full org directory user picker (Graph) + JIT-stub Entra group members</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Purpose: let owners/admins pick any user in the Entra tenant, not only people who have already signed into the app.
-Why deferred: WP2b picker uses GET /api/users (JIT-provisioned DB rows only) to avoid Graph scopes and pending-grant edge cases.
-Steps: (1) Graph User.Read.All or equivalent search; (2) typeahead against tenant directory; (3) on grant to never-seen user, either JIT stub user or pending grant resolved at first login; (4) document privacy/consent.</t>
+          <t>Purpose: let owners/admins pick any user in the Entra tenant, not only people who have already signed into the app, AND surface Entra group members that have never signed in yet.
+Why deferred (pre-4.21): WP2b picker used GET /api/users (JIT-provisioned DB rows only) to avoid Graph scopes and pending-grant edge cases. WBS 4.20 sync skipped Entra group members with no local user row for the same reason.
+Delivered (PR feat/wbs-4.21-directory-picker): (1) Graph User.Read.All permission documented alongside 4.20's GroupMember.Read.All; (2) GET /api/users/directory tenant-directory typeahead + POST /api/users/from-entra JIT-stub endpoint (both authenticated, not admin-only; from-entra validates the OID against Graph before insert to prevent forgery); (3) commands/entra_group_sync.py now stubs previously-skipped members via list_users_by_oids chunked at 15; (4) upsert-at-first-login already exercised by existing EntraOIDCProvider test; (5) InviteFromDirectoryDialog wired into Groups admin page and ShareSheet, "Never signed in" badge on stub users; (6) AUTH.md § Directory picker + SHARING.md updated; env vars documented (no new env — reuses Entra client credentials).</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Directory-backed share/group member picker</t>
-        </is>
-      </c>
-      <c r="F64" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
+          <t>Directory-backed share/group member picker; Entra group members visible before first login</t>
+        </is>
+      </c>
+      <c r="F64" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G64" s="16" t="inlineStr">
@@ -6194,10 +6192,10 @@
         </is>
       </c>
       <c r="I64" s="17" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="J64" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K64" s="17" t="n"/>
       <c r="L64" s="18" t="n">
@@ -6213,17 +6211,17 @@
       <c r="P64" s="3" t="n"/>
       <c r="Q64" s="3" t="inlineStr">
         <is>
-          <t>Can share with a colleague who has never opened the app yet; first login attaches access</t>
+          <t>Admin/owner can share with any tenant colleague (never opened app) + WBS 4.20 sync stops skipping unknown members</t>
         </is>
       </c>
       <c r="R64" s="3" t="inlineStr">
         <is>
-          <t>Pairs with 4.20; keep DB-user picker as fallback</t>
+          <t>Pairs with 4.20; keep DB-user picker as fallback; JIT-stub semantics touch sync + share flow — one spec, one PR</t>
         </is>
       </c>
       <c r="S64" s="3" t="inlineStr">
         <is>
-          <t>GET /api/users today = signed-in only</t>
+          <t>GET /api/users today = signed-in only; entra_group_sync.py members_skipped_unknown counter</t>
         </is>
       </c>
     </row>
@@ -6309,28 +6307,29 @@
     <row r="66" ht="75" customHeight="1">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.23</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>WP3 — Frontend Map + White-label</t>
+          <t>Carry-forward / Sharing Follow-through</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>WP3 kickoff</t>
+          <t>Entra ID group-membership webhooks (Graph change notifications)</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Purpose: start white-label work only after identity is on main.
-Steps: create wp-3-white-label; confirm Model A brand loads once at app startup (not per request).</t>
+          <t>Purpose: replace WBS 4.20's polling loop (default 15 min) with live push-based updates from Microsoft Graph so ACL changes propagate within seconds.
+Why deferred from 4.20: needs a publicly-reachable HTTPS callback URL, HMAC/clientState validation, subscription lifecycle (create + auto-renewal every ~3 days per Graph limit), replay-dedupe, and rotation of the validation token — each with its own security review. Bundling with 4.20 would ~double that PR's risk surface.
+Steps: (1) design spec covering callback URL, clientState secret storage, subscription table schema, renewal cron; (2) POST /api/graph/webhook endpoint with validation-token handshake + subscribe/renew/delete lifecycle; (3) event handler that maps 'groupMembers changed' events to a scoped sync_entra_groups(group_id=...) submission; (4) background job that renews subscriptions with lead time before ~3-day expiry; (5) fall back cleanly to the periodic loop when the webhook subscription is missing or invalid; (6) docs (AUTH.md § Entra group sync/webhooks) + admin UI status pill for subscription health.</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Branch</t>
+          <t>Live push-based Entra group-membership sync</t>
         </is>
       </c>
       <c r="F66" s="22" t="inlineStr">
@@ -6338,21 +6337,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G66" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G66" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
-          <t>4.19</t>
+          <t>4.20</t>
         </is>
       </c>
       <c r="I66" s="17" t="n">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="J66" s="17" t="n">
-        <v>0.25</v>
+        <v>4</v>
       </c>
       <c r="K66" s="17" t="n"/>
       <c r="L66" s="18" t="n">
@@ -6360,32 +6359,32 @@
       </c>
       <c r="M66" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
-        </is>
-      </c>
-      <c r="N66" s="19" t="n">
-        <v>46253</v>
-      </c>
-      <c r="O66" s="19" t="n">
-        <v>46253</v>
-      </c>
+          <t>Backend Engineer</t>
+        </is>
+      </c>
+      <c r="N66" s="3" t="n"/>
+      <c r="O66" s="3" t="n"/>
       <c r="P66" s="3" t="n"/>
       <c r="Q66" s="3" t="inlineStr">
         <is>
-          <t>Branch created after WP2b merge (or after WP2 if WP2b still open — prefer after 4.19)</t>
+          <t>Entra group membership changes reflect in ACL within seconds (not up to 15 min); subscriptions auto-renew before expiry; missing/invalid subscription silently falls back to the existing periodic loop</t>
         </is>
       </c>
       <c r="R66" s="3" t="inlineStr">
         <is>
-          <t>Optional admin brand UI needs WP2 roles; do not mix with wp-2b-sharing</t>
-        </is>
-      </c>
-      <c r="S66" s="3" t="inlineStr"/>
+          <t>Do NOT bundle with 4.20 — subscription lifecycle deserves its own PR + security review</t>
+        </is>
+      </c>
+      <c r="S66" s="3" t="inlineStr">
+        <is>
+          <t>commands/entra_group_sync.py periodic loop; docs/AUTH.md § Entra group sync (WBS 4.20)</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="75" customHeight="1">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -6395,18 +6394,18 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>Produce docs/FRONTEND_MAP.md</t>
+          <t>WP3 kickoff</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Purpose: make every future UI change locatable without archaeology.
-Steps: for each auth and dashboard route, document page → component tree, stores/hooks/API calls, shared layout, component catalog, and a where-do-I-change-X table.</t>
+          <t>Purpose: start white-label work only after identity is on main.
+Steps: create wp-3-white-label; confirm Model A brand loads once at app startup (not per request).</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>docs/FRONTEND_MAP.md</t>
+          <t>Branch</t>
         </is>
       </c>
       <c r="F67" s="22" t="inlineStr">
@@ -6421,14 +6420,14 @@
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.19</t>
         </is>
       </c>
       <c r="I67" s="17" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="J67" s="17" t="n">
-        <v>2.5</v>
+        <v>0.25</v>
       </c>
       <c r="K67" s="17" t="n"/>
       <c r="L67" s="18" t="n">
@@ -6443,21 +6442,25 @@
         <v>46253</v>
       </c>
       <c r="O67" s="19" t="n">
-        <v>46255</v>
+        <v>46253</v>
       </c>
       <c r="P67" s="3" t="n"/>
       <c r="Q67" s="3" t="inlineStr">
         <is>
-          <t>Map covers every route with data flow + backend calls</t>
-        </is>
-      </c>
-      <c r="R67" s="3" t="inlineStr"/>
+          <t>Branch created after WP2b merge (or after WP2 if WP2b still open — prefer after 4.19)</t>
+        </is>
+      </c>
+      <c r="R67" s="3" t="inlineStr">
+        <is>
+          <t>Optional admin brand UI needs WP2 roles; do not mix with wp-2b-sharing</t>
+        </is>
+      </c>
       <c r="S67" s="3" t="inlineStr"/>
     </row>
     <row r="68" ht="75" customHeight="1">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -6467,18 +6470,18 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>BrandConfig schema + loader</t>
+          <t>Produce docs/FRONTEND_MAP.md</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Purpose: drive app name, logos, favicon, colours, font, and support URL from config so clients do not need a rebuild.
-Steps: define BrandConfig schema; load from BRAND_CONFIG_PATH or /config/brand at startup under Model A.</t>
+          <t>Purpose: make every future UI change locatable without archaeology.
+Steps: for each auth and dashboard route, document page → component tree, stores/hooks/API calls, shared layout, component catalog, and a where-do-I-change-X table.</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>BrandConfig type + loader</t>
+          <t>docs/FRONTEND_MAP.md</t>
         </is>
       </c>
       <c r="F68" s="22" t="inlineStr">
@@ -6486,9 +6489,9 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G68" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G68" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H68" s="3" t="inlineStr">
@@ -6497,10 +6500,10 @@
         </is>
       </c>
       <c r="I68" s="17" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="J68" s="17" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="K68" s="17" t="n"/>
       <c r="L68" s="18" t="n">
@@ -6508,19 +6511,19 @@
       </c>
       <c r="M68" s="3" t="inlineStr">
         <is>
-          <t>Full-stack</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N68" s="19" t="n">
+        <v>46253</v>
+      </c>
+      <c r="O68" s="19" t="n">
         <v>46255</v>
-      </c>
-      <c r="O68" s="19" t="n">
-        <v>46256</v>
       </c>
       <c r="P68" s="3" t="n"/>
       <c r="Q68" s="3" t="inlineStr">
         <is>
-          <t>Config loads without a rebuild</t>
+          <t>Map covers every route with data flow + backend calls</t>
         </is>
       </c>
       <c r="R68" s="3" t="inlineStr"/>
@@ -6529,7 +6532,7 @@
     <row r="69" ht="75" customHeight="1">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>5.2</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -6539,18 +6542,18 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>Runtime theme injection (CSS variables)</t>
+          <t>BrandConfig schema + loader</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Purpose: apply BrandConfig at runtime to CSS variables for light and dark themes.
-Steps: map colours to :root / dark variants; replace hardcoded title and /logo.svg; use the brand inventory in LICENSE_COMPLIANCE §8; demonstrate two brands from one build.</t>
+          <t>Purpose: drive app name, logos, favicon, colours, font, and support URL from config so clients do not need a rebuild.
+Steps: define BrandConfig schema; load from BRAND_CONFIG_PATH or /config/brand at startup under Model A.</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Runtime theming</t>
+          <t>BrandConfig type + loader</t>
         </is>
       </c>
       <c r="F69" s="22" t="inlineStr">
@@ -6565,14 +6568,14 @@
       </c>
       <c r="H69" s="3" t="inlineStr">
         <is>
-          <t>5.2</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="I69" s="17" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="J69" s="17" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="K69" s="17" t="n"/>
       <c r="L69" s="18" t="n">
@@ -6580,19 +6583,19 @@
       </c>
       <c r="M69" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>Full-stack</t>
         </is>
       </c>
       <c r="N69" s="19" t="n">
+        <v>46255</v>
+      </c>
+      <c r="O69" s="19" t="n">
         <v>46256</v>
-      </c>
-      <c r="O69" s="19" t="n">
-        <v>46259</v>
       </c>
       <c r="P69" s="3" t="n"/>
       <c r="Q69" s="3" t="inlineStr">
         <is>
-          <t>Two visibly different brands from the same build; no code edit to rebrand</t>
+          <t>Config loads without a rebuild</t>
         </is>
       </c>
       <c r="R69" s="3" t="inlineStr"/>
@@ -6601,7 +6604,7 @@
     <row r="70" ht="75" customHeight="1">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>5.4</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -6611,18 +6614,18 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>themes/ presets + add-client procedure</t>
+          <t>Runtime theme injection (CSS variables)</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>Purpose: make “add a client theme” a documented drop-in of config + assets.
-Steps: ship at least two presets under themes/; write the operator procedure (no rebuild).</t>
+          <t>Purpose: apply BrandConfig at runtime to CSS variables for light and dark themes.
+Steps: map colours to :root / dark variants; replace hardcoded title and /logo.svg; use the brand inventory in LICENSE_COMPLIANCE §8; demonstrate two brands from one build.</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>themes/ + docs procedure</t>
+          <t>Runtime theming</t>
         </is>
       </c>
       <c r="F70" s="22" t="inlineStr">
@@ -6630,21 +6633,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G70" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G70" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>5.3</t>
+          <t>5.2</t>
         </is>
       </c>
       <c r="I70" s="17" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="J70" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K70" s="17" t="n"/>
       <c r="L70" s="18" t="n">
@@ -6656,15 +6659,15 @@
         </is>
       </c>
       <c r="N70" s="19" t="n">
+        <v>46256</v>
+      </c>
+      <c r="O70" s="19" t="n">
         <v>46259</v>
-      </c>
-      <c r="O70" s="19" t="n">
-        <v>46260</v>
       </c>
       <c r="P70" s="3" t="n"/>
       <c r="Q70" s="3" t="inlineStr">
         <is>
-          <t>Documented procedure produces two different brands from one build</t>
+          <t>Two visibly different brands from the same build; no code edit to rebrand</t>
         </is>
       </c>
       <c r="R70" s="3" t="inlineStr"/>
@@ -6673,7 +6676,7 @@
     <row r="71" ht="75" customHeight="1">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>5.4</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -6683,18 +6686,18 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Optional admin BrandConfig UI</t>
+          <t>themes/ presets + add-client procedure</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Purpose (optional): let admins edit BrandConfig live without redeploying.
-Steps: admin-only settings screen gated by WP2 roles; persist and hot-apply theme.</t>
+          <t>Purpose: make “add a client theme” a documented drop-in of config + assets.
+Steps: ship at least two presets under themes/; write the operator procedure (no rebuild).</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Admin brand settings UI</t>
+          <t>themes/ + docs procedure</t>
         </is>
       </c>
       <c r="F71" s="22" t="inlineStr">
@@ -6702,21 +6705,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G71" s="24" t="inlineStr">
-        <is>
-          <t>Low</t>
+      <c r="G71" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
-          <t>5.3,4.5</t>
+          <t>5.3</t>
         </is>
       </c>
       <c r="I71" s="17" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="J71" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K71" s="17" t="n"/>
       <c r="L71" s="18" t="n">
@@ -6728,28 +6731,24 @@
         </is>
       </c>
       <c r="N71" s="19" t="n">
+        <v>46259</v>
+      </c>
+      <c r="O71" s="19" t="n">
         <v>46260</v>
-      </c>
-      <c r="O71" s="19" t="n">
-        <v>46262</v>
       </c>
       <c r="P71" s="3" t="n"/>
       <c r="Q71" s="3" t="inlineStr">
         <is>
-          <t>Admin can edit brand without redeploy (optional acceptance)</t>
-        </is>
-      </c>
-      <c r="R71" s="3" t="inlineStr">
-        <is>
-          <t>Optional per master plan</t>
-        </is>
-      </c>
+          <t>Documented procedure produces two different brands from one build</t>
+        </is>
+      </c>
+      <c r="R71" s="3" t="inlineStr"/>
       <c r="S71" s="3" t="inlineStr"/>
     </row>
     <row r="72" ht="75" customHeight="1">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>5.5</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -6759,18 +6758,18 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>WP3 verification + review stop</t>
+          <t>Optional admin BrandConfig UI</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>Purpose: close white-label only when map + config branding acceptance criteria pass.
-Steps: verify ACs; PR; human review; do not mix WP5 on the same branch.</t>
+          <t>Purpose (optional): let admins edit BrandConfig live without redeploying.
+Steps: admin-only settings screen gated by WP2 roles; persist and hot-apply theme.</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>Merged WP3</t>
+          <t>Admin brand settings UI</t>
         </is>
       </c>
       <c r="F72" s="22" t="inlineStr">
@@ -6778,21 +6777,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G72" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G72" s="23" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
-          <t>5.1,5.4</t>
+          <t>5.3,4.5</t>
         </is>
       </c>
       <c r="I72" s="17" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="J72" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K72" s="17" t="n"/>
       <c r="L72" s="18" t="n">
@@ -6800,49 +6799,53 @@
       </c>
       <c r="M72" s="3" t="inlineStr">
         <is>
-          <t>Engineering Lead</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N72" s="19" t="n">
+        <v>46260</v>
+      </c>
+      <c r="O72" s="19" t="n">
         <v>46262</v>
-      </c>
-      <c r="O72" s="19" t="n">
-        <v>46263</v>
       </c>
       <c r="P72" s="3" t="n"/>
       <c r="Q72" s="3" t="inlineStr">
         <is>
-          <t>All WP3 acceptance criteria pass</t>
-        </is>
-      </c>
-      <c r="R72" s="3" t="inlineStr"/>
+          <t>Admin can edit brand without redeploy (optional acceptance)</t>
+        </is>
+      </c>
+      <c r="R72" s="3" t="inlineStr">
+        <is>
+          <t>Optional per master plan</t>
+        </is>
+      </c>
       <c r="S72" s="3" t="inlineStr"/>
     </row>
     <row r="73" ht="75" customHeight="1">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>5.6</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>WP4 — Backend/API Documentation</t>
+          <t>WP3 — Frontend Map + White-label</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>WP4 kickoff (can parallel early)</t>
+          <t>WP3 verification + review stop</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Purpose: start the backend architecture map as documentation-only, low-risk work.
-Steps: create wp-4-backend-map; prefer starting after WP2 so auth docs match reality; can begin after WP0 if staffed in parallel.</t>
+          <t>Purpose: close white-label only when map + config branding acceptance criteria pass.
+Steps: verify ACs; PR; human review; do not mix WP5 on the same branch.</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Branch</t>
+          <t>Merged WP3</t>
         </is>
       </c>
       <c r="F73" s="22" t="inlineStr">
@@ -6850,21 +6853,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G73" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G73" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H73" s="3" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>5.1,5.4</t>
         </is>
       </c>
       <c r="I73" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="J73" s="17" t="n">
         <v>1</v>
-      </c>
-      <c r="J73" s="17" t="n">
-        <v>0.25</v>
       </c>
       <c r="K73" s="17" t="n"/>
       <c r="L73" s="18" t="n">
@@ -6872,439 +6875,475 @@
       </c>
       <c r="M73" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Engineering Lead</t>
         </is>
       </c>
       <c r="N73" s="19" t="n">
-        <v>46253</v>
+        <v>46262</v>
       </c>
       <c r="O73" s="19" t="n">
-        <v>46253</v>
+        <v>46263</v>
       </c>
       <c r="P73" s="3" t="n"/>
       <c r="Q73" s="3" t="inlineStr">
         <is>
-          <t>Docs branch ready</t>
-        </is>
-      </c>
-      <c r="R73" s="3" t="inlineStr">
-        <is>
-          <t>Better after WP2 for accurate auth sections</t>
-        </is>
-      </c>
+          <t>All WP3 acceptance criteria pass</t>
+        </is>
+      </c>
+      <c r="R73" s="3" t="inlineStr"/>
       <c r="S73" s="3" t="inlineStr"/>
     </row>
     <row r="74" ht="75" customHeight="1">
       <c r="A74" s="3" t="inlineStr">
         <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>WP4 — Backend/API Documentation</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>WP4 kickoff (can parallel early)</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: start the backend architecture map as documentation-only, low-risk work.
+Steps: create wp-4-backend-map; prefer starting after WP2 so auth docs match reality; can begin after WP0 if staffed in parallel.</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="F74" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G74" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>1.11</t>
+        </is>
+      </c>
+      <c r="I74" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J74" s="17" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K74" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L74" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M74" s="3" t="inlineStr">
+        <is>
+          <t>Backend Engineer</t>
+        </is>
+      </c>
+      <c r="N74" s="19" t="n">
+        <v>46253</v>
+      </c>
+      <c r="O74" s="19" t="n">
+        <v>46253</v>
+      </c>
+      <c r="P74" s="19" t="n">
+        <v>46294</v>
+      </c>
+      <c r="Q74" s="3" t="inlineStr">
+        <is>
+          <t>Docs branch ready</t>
+        </is>
+      </c>
+      <c r="R74" s="3" t="inlineStr">
+        <is>
+          <t>Better after WP2 for accurate auth sections</t>
+        </is>
+      </c>
+      <c r="S74" s="3" t="inlineStr">
+        <is>
+          <t>PR #55</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="75" customHeight="1">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
           <t>6.1</t>
         </is>
       </c>
-      <c r="B74" s="3" t="inlineStr">
+      <c r="B75" s="3" t="inlineStr">
         <is>
           <t>WP4 — Backend/API Documentation</t>
         </is>
       </c>
-      <c r="C74" s="3" t="inlineStr">
+      <c r="C75" s="3" t="inlineStr">
         <is>
           <t>Router catalog (all endpoints)</t>
         </is>
       </c>
-      <c r="D74" s="3" t="inlineStr">
+      <c r="D75" s="3" t="inlineStr">
         <is>
           <t>Purpose: catalogue every HTTP endpoint with method, path, models, auth requirement, and service/domain call.
 Steps: walk all routers; document consistently; update after WP2 auth lands.</t>
         </is>
       </c>
-      <c r="E74" s="3" t="inlineStr">
+      <c r="E75" s="3" t="inlineStr">
         <is>
           <t>BACKEND_MAP.md routers section</t>
         </is>
       </c>
-      <c r="F74" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G74" s="21" t="inlineStr">
+      <c r="F75" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G75" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H74" s="3" t="inlineStr">
+      <c r="H75" s="3" t="inlineStr">
         <is>
           <t>6.0</t>
         </is>
       </c>
-      <c r="I74" s="17" t="n">
+      <c r="I75" s="17" t="n">
         <v>16</v>
       </c>
-      <c r="J74" s="17" t="n">
+      <c r="J75" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="K74" s="17" t="n"/>
-      <c r="L74" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M74" s="3" t="inlineStr">
+      <c r="K75" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="L75" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M75" s="3" t="inlineStr">
         <is>
           <t>Backend Engineer</t>
         </is>
       </c>
-      <c r="N74" s="19" t="n">
+      <c r="N75" s="19" t="n">
         <v>46253</v>
       </c>
-      <c r="O74" s="19" t="n">
+      <c r="O75" s="19" t="n">
         <v>46255</v>
       </c>
-      <c r="P74" s="3" t="n"/>
-      <c r="Q74" s="3" t="inlineStr">
+      <c r="P75" s="19" t="n">
+        <v>46294</v>
+      </c>
+      <c r="Q75" s="3" t="inlineStr">
         <is>
           <t>Every endpoint documented with auth + models</t>
         </is>
       </c>
-      <c r="R74" s="3" t="inlineStr"/>
-      <c r="S74" s="3" t="inlineStr"/>
-    </row>
-    <row r="75" ht="75" customHeight="1">
-      <c r="A75" s="3" t="inlineStr">
+      <c r="R75" s="3" t="inlineStr"/>
+      <c r="S75" s="3" t="inlineStr">
+        <is>
+          <t>PR #55 docs/BACKEND_MAP.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="75" customHeight="1">
+      <c r="A76" s="3" t="inlineStr">
         <is>
           <t>6.2</t>
         </is>
       </c>
-      <c r="B75" s="3" t="inlineStr">
+      <c r="B76" s="3" t="inlineStr">
         <is>
           <t>WP4 — Backend/API Documentation</t>
         </is>
       </c>
-      <c r="C75" s="3" t="inlineStr">
+      <c r="C76" s="3" t="inlineStr">
         <is>
           <t>Domain model + graph + data layer maps</t>
         </is>
       </c>
-      <c r="D75" s="3" t="inlineStr">
+      <c r="D76" s="3" t="inlineStr">
         <is>
           <t>Purpose: document ObjectModel patterns, LangGraph flows, repository usage, migrations, and SurrealDB features in use.
 Steps: catalogue models/relationships; map each graph’s inputs/steps/outputs; explain repository call-site pattern and migrations.</t>
         </is>
       </c>
-      <c r="E75" s="3" t="inlineStr">
+      <c r="E76" s="3" t="inlineStr">
         <is>
           <t>BACKEND_MAP.md domain/graphs/data</t>
         </is>
       </c>
-      <c r="F75" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G75" s="21" t="inlineStr">
+      <c r="F76" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G76" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H75" s="3" t="inlineStr">
+      <c r="H76" s="3" t="inlineStr">
         <is>
           <t>6.1</t>
         </is>
       </c>
-      <c r="I75" s="17" t="n">
+      <c r="I76" s="17" t="n">
         <v>16</v>
       </c>
-      <c r="J75" s="17" t="n">
+      <c r="J76" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="K75" s="17" t="n"/>
-      <c r="L75" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M75" s="3" t="inlineStr">
+      <c r="K76" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="L76" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M76" s="3" t="inlineStr">
         <is>
           <t>Backend Engineer</t>
         </is>
       </c>
-      <c r="N75" s="19" t="n">
+      <c r="N76" s="19" t="n">
         <v>46255</v>
       </c>
-      <c r="O75" s="19" t="n">
+      <c r="O76" s="19" t="n">
         <v>46259</v>
       </c>
-      <c r="P75" s="3" t="n"/>
-      <c r="Q75" s="3" t="inlineStr">
+      <c r="P76" s="19" t="n">
+        <v>46294</v>
+      </c>
+      <c r="Q76" s="3" t="inlineStr">
         <is>
           <t>Every domain model and graph documented</t>
         </is>
       </c>
-      <c r="R75" s="3" t="inlineStr"/>
-      <c r="S75" s="3" t="inlineStr"/>
-    </row>
-    <row r="76" ht="75" customHeight="1">
-      <c r="A76" s="3" t="inlineStr">
+      <c r="R76" s="3" t="inlineStr"/>
+      <c r="S76" s="3" t="inlineStr">
+        <is>
+          <t>PR #55 docs/BACKEND_MAP.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="75" customHeight="1">
+      <c r="A77" s="3" t="inlineStr">
         <is>
           <t>6.3</t>
         </is>
       </c>
-      <c r="B76" s="3" t="inlineStr">
+      <c r="B77" s="3" t="inlineStr">
         <is>
           <t>WP4 — Backend/API Documentation</t>
         </is>
       </c>
-      <c r="C76" s="3" t="inlineStr">
+      <c r="C77" s="3" t="inlineStr">
         <is>
           <t>Jobs, config/secrets, how-to playbooks</t>
         </is>
       </c>
-      <c r="D76" s="3" t="inlineStr">
+      <c r="D77" s="3" t="inlineStr">
         <is>
           <t>Purpose: finish the operator/engineer map with jobs, env vars, and five how-to-add playbooks.
 Steps: document surreal-commands; env/secrets; playbooks for endpoint, model+migration, provider, job, source type; reconcile with existing change-playbooks.md.</t>
         </is>
       </c>
-      <c r="E76" s="3" t="inlineStr">
+      <c r="E77" s="3" t="inlineStr">
         <is>
           <t>BACKEND_MAP.md complete</t>
         </is>
       </c>
-      <c r="F76" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G76" s="21" t="inlineStr">
+      <c r="F77" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G77" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H76" s="3" t="inlineStr">
+      <c r="H77" s="3" t="inlineStr">
         <is>
           <t>6.2</t>
         </is>
       </c>
-      <c r="I76" s="17" t="n">
+      <c r="I77" s="17" t="n">
         <v>12</v>
       </c>
-      <c r="J76" s="17" t="n">
+      <c r="J77" s="17" t="n">
         <v>1.5</v>
       </c>
-      <c r="K76" s="17" t="n"/>
-      <c r="L76" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M76" s="3" t="inlineStr">
+      <c r="K77" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="L77" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M77" s="3" t="inlineStr">
         <is>
           <t>Backend Engineer</t>
         </is>
       </c>
-      <c r="N76" s="19" t="n">
+      <c r="N77" s="19" t="n">
         <v>46259</v>
       </c>
-      <c r="O76" s="19" t="n">
+      <c r="O77" s="19" t="n">
         <v>46260</v>
       </c>
-      <c r="P76" s="3" t="n"/>
-      <c r="Q76" s="3" t="inlineStr">
+      <c r="P77" s="19" t="n">
+        <v>46294</v>
+      </c>
+      <c r="Q77" s="3" t="inlineStr">
         <is>
           <t>Five how-to playbooks present and accurate</t>
         </is>
       </c>
-      <c r="R76" s="3" t="inlineStr"/>
-      <c r="S76" s="3" t="inlineStr"/>
-    </row>
-    <row r="77" ht="75" customHeight="1">
-      <c r="A77" s="3" t="inlineStr">
+      <c r="R77" s="3" t="inlineStr"/>
+      <c r="S77" s="3" t="inlineStr">
+        <is>
+          <t>PR #55 docs/BACKEND_MAP.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="75" customHeight="1">
+      <c r="A78" s="3" t="inlineStr">
         <is>
           <t>6.4</t>
         </is>
       </c>
-      <c r="B77" s="3" t="inlineStr">
+      <c r="B78" s="3" t="inlineStr">
         <is>
           <t>WP4 — Backend/API Documentation</t>
         </is>
       </c>
-      <c r="C77" s="3" t="inlineStr">
+      <c r="C78" s="3" t="inlineStr">
         <is>
           <t>WP4 review stop</t>
         </is>
       </c>
-      <c r="D77" s="3" t="inlineStr">
+      <c r="D78" s="3" t="inlineStr">
         <is>
           <t>Purpose: peer-review the map for accuracy and merge.
 Steps: review against live code; fix gaps; merge; confirm a new engineer can locate changes using only BACKEND_MAP.</t>
         </is>
       </c>
-      <c r="E77" s="3" t="inlineStr">
+      <c r="E78" s="3" t="inlineStr">
         <is>
           <t>docs/BACKEND_MAP.md on main</t>
         </is>
       </c>
-      <c r="F77" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G77" s="21" t="inlineStr">
+      <c r="F78" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G78" s="21" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="H77" s="3" t="inlineStr">
+      <c r="H78" s="3" t="inlineStr">
         <is>
           <t>6.3</t>
         </is>
       </c>
-      <c r="I77" s="17" t="n">
+      <c r="I78" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="J77" s="17" t="n">
+      <c r="J78" s="17" t="n">
         <v>0.5</v>
       </c>
-      <c r="K77" s="17" t="n"/>
-      <c r="L77" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M77" s="3" t="inlineStr">
+      <c r="K78" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="L78" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M78" s="3" t="inlineStr">
         <is>
           <t>Engineering Lead</t>
         </is>
       </c>
-      <c r="N77" s="19" t="n">
+      <c r="N78" s="19" t="n">
         <v>46260</v>
       </c>
-      <c r="O77" s="19" t="n">
+      <c r="O78" s="19" t="n">
         <v>46261</v>
       </c>
-      <c r="P77" s="3" t="n"/>
-      <c r="Q77" s="3" t="inlineStr">
+      <c r="P78" s="19" t="n">
+        <v>46294</v>
+      </c>
+      <c r="Q78" s="3" t="inlineStr">
         <is>
           <t>New engineer can locate changes using only this doc</t>
         </is>
       </c>
-      <c r="R77" s="3" t="inlineStr"/>
-      <c r="S77" s="3" t="inlineStr"/>
-    </row>
-    <row r="78" ht="75" customHeight="1">
-      <c r="A78" s="3" t="inlineStr">
+      <c r="R78" s="3" t="inlineStr"/>
+      <c r="S78" s="3" t="inlineStr">
+        <is>
+          <t>PR #55</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="75" customHeight="1">
+      <c r="A79" s="3" t="inlineStr">
         <is>
           <t>7.0</t>
         </is>
       </c>
-      <c r="B78" s="3" t="inlineStr">
+      <c r="B79" s="3" t="inlineStr">
         <is>
           <t>WP5 — External Source Connectors</t>
         </is>
       </c>
-      <c r="C78" s="3" t="inlineStr">
+      <c r="C79" s="3" t="inlineStr">
         <is>
           <t>WP5 kickoff</t>
         </is>
       </c>
-      <c r="D78" s="3" t="inlineStr">
+      <c r="D79" s="3" t="inlineStr">
         <is>
           <t>Purpose: design connectors that feed the existing ingestion pipeline instead of reinventing extraction.
 Steps: create wp-5-connectors; draft SourceConnector interface; confirm hard dependency on WP2 for per-user OAuth tokens.</t>
         </is>
       </c>
-      <c r="E78" s="3" t="inlineStr">
+      <c r="E79" s="3" t="inlineStr">
         <is>
           <t>Branch + design note</t>
         </is>
       </c>
-      <c r="F78" s="22" t="inlineStr">
+      <c r="F79" s="22" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="G78" s="16" t="inlineStr">
+      <c r="G79" s="16" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H78" s="3" t="inlineStr">
+      <c r="H79" s="3" t="inlineStr">
         <is>
           <t>4.10</t>
         </is>
       </c>
-      <c r="I78" s="17" t="n">
+      <c r="I79" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="J78" s="17" t="n">
+      <c r="J79" s="17" t="n">
         <v>0.5</v>
-      </c>
-      <c r="K78" s="17" t="n"/>
-      <c r="L78" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="M78" s="3" t="inlineStr">
-        <is>
-          <t>Engineer</t>
-        </is>
-      </c>
-      <c r="N78" s="19" t="n">
-        <v>46266</v>
-      </c>
-      <c r="O78" s="19" t="n">
-        <v>46266</v>
-      </c>
-      <c r="P78" s="3" t="n"/>
-      <c r="Q78" s="3" t="inlineStr">
-        <is>
-          <t>Design reuses content-core + graphs/source.py</t>
-        </is>
-      </c>
-      <c r="R78" s="3" t="inlineStr">
-        <is>
-          <t>Blocked until WP2 users/tokens exist</t>
-        </is>
-      </c>
-      <c r="S78" s="3" t="inlineStr"/>
-    </row>
-    <row r="79" ht="75" customHeight="1">
-      <c r="A79" s="3" t="inlineStr">
-        <is>
-          <t>7.1</t>
-        </is>
-      </c>
-      <c r="B79" s="3" t="inlineStr">
-        <is>
-          <t>WP5 — External Source Connectors</t>
-        </is>
-      </c>
-      <c r="C79" s="3" t="inlineStr">
-        <is>
-          <t>SourceConnector interface + bulk job fan-out</t>
-        </is>
-      </c>
-      <c r="D79" s="3" t="inlineStr">
-        <is>
-          <t>Purpose: one “add location” action becomes N document jobs with per-doc progress and partial failure tolerance.
-Steps: define authenticate/list_documents/fetch_document; extend source_commands for fan-out; ensure one bad file does not abort the batch.</t>
-        </is>
-      </c>
-      <c r="E79" s="3" t="inlineStr">
-        <is>
-          <t>Connector API + bulk command</t>
-        </is>
-      </c>
-      <c r="F79" s="22" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G79" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="H79" s="3" t="inlineStr">
-        <is>
-          <t>7.0</t>
-        </is>
-      </c>
-      <c r="I79" s="17" t="n">
-        <v>24</v>
-      </c>
-      <c r="J79" s="17" t="n">
-        <v>3</v>
       </c>
       <c r="K79" s="17" t="n"/>
       <c r="L79" s="18" t="n">
@@ -7312,28 +7351,32 @@
       </c>
       <c r="M79" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N79" s="19" t="n">
         <v>46266</v>
       </c>
       <c r="O79" s="19" t="n">
-        <v>46269</v>
+        <v>46266</v>
       </c>
       <c r="P79" s="3" t="n"/>
       <c r="Q79" s="3" t="inlineStr">
         <is>
-          <t>Single failure does not abort batch; progress per document</t>
-        </is>
-      </c>
-      <c r="R79" s="3" t="inlineStr"/>
+          <t>Design reuses content-core + graphs/source.py</t>
+        </is>
+      </c>
+      <c r="R79" s="3" t="inlineStr">
+        <is>
+          <t>Blocked until WP2 users/tokens exist</t>
+        </is>
+      </c>
       <c r="S79" s="3" t="inlineStr"/>
     </row>
     <row r="80" ht="75" customHeight="1">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>7.2</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
@@ -7343,18 +7386,18 @@
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>SharePoint connector (Microsoft Graph)</t>
+          <t>SourceConnector interface + bulk job fan-out</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Purpose: let an Entra-signed-in user pull an entire SharePoint folder into chat-able sources.
-Steps: OAuth on behalf of the user; least-privilege Sites/Files read scopes; enumerate folder; download supported files into existing ingestion; document admin consent.</t>
+          <t>Purpose: one “add location” action becomes N document jobs with per-doc progress and partial failure tolerance.
+Steps: define authenticate/list_documents/fetch_document; extend source_commands for fan-out; ensure one bad file does not abort the batch.</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>SharePointConnector</t>
+          <t>Connector API + bulk command</t>
         </is>
       </c>
       <c r="F80" s="22" t="inlineStr">
@@ -7369,14 +7412,14 @@
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>7.1,4.7</t>
+          <t>7.0</t>
         </is>
       </c>
       <c r="I80" s="17" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="J80" s="17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K80" s="17" t="n"/>
       <c r="L80" s="18" t="n">
@@ -7388,15 +7431,15 @@
         </is>
       </c>
       <c r="N80" s="19" t="n">
+        <v>46266</v>
+      </c>
+      <c r="O80" s="19" t="n">
         <v>46269</v>
-      </c>
-      <c r="O80" s="19" t="n">
-        <v>46275</v>
       </c>
       <c r="P80" s="3" t="n"/>
       <c r="Q80" s="3" t="inlineStr">
         <is>
-          <t>User connects SharePoint, picks folder, pulls all supported docs</t>
+          <t>Single failure does not abort batch; progress per document</t>
         </is>
       </c>
       <c r="R80" s="3" t="inlineStr"/>
@@ -7405,7 +7448,7 @@
     <row r="81" ht="75" customHeight="1">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>7.2</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -7415,18 +7458,18 @@
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>Generic DMS / multi-doc link connector</t>
+          <t>SharePoint connector (Microsoft Graph)</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Purpose: support folder URLs / IDs that resolve to many documents, with an extension point for other DMS systems.
-Steps: implement base multi-doc connector; keep the SourceConnector interface as the only required surface for new connectors.</t>
+          <t>Purpose: let an Entra-signed-in user pull an entire SharePoint folder into chat-able sources.
+Steps: OAuth on behalf of the user; least-privilege Sites/Files read scopes; enumerate folder; download supported files into existing ingestion; document admin consent.</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>Generic multi-doc connector</t>
+          <t>SharePointConnector</t>
         </is>
       </c>
       <c r="F81" s="22" t="inlineStr">
@@ -7434,21 +7477,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G81" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G81" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>7.1,4.7</t>
         </is>
       </c>
       <c r="I81" s="17" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="J81" s="17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K81" s="17" t="n"/>
       <c r="L81" s="18" t="n">
@@ -7460,7 +7503,7 @@
         </is>
       </c>
       <c r="N81" s="19" t="n">
-        <v>46273</v>
+        <v>46269</v>
       </c>
       <c r="O81" s="19" t="n">
         <v>46275</v>
@@ -7468,7 +7511,7 @@
       <c r="P81" s="3" t="n"/>
       <c r="Q81" s="3" t="inlineStr">
         <is>
-          <t>New connector = implement interface only</t>
+          <t>User connects SharePoint, picks folder, pulls all supported docs</t>
         </is>
       </c>
       <c r="R81" s="3" t="inlineStr"/>
@@ -7477,7 +7520,7 @@
     <row r="82" ht="75" customHeight="1">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>7.4</t>
+          <t>7.3</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -7487,18 +7530,18 @@
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>Encrypted per-user token storage</t>
+          <t>Generic DMS / multi-doc link connector</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>Purpose: store connector OAuth tokens encrypted per user using existing encryption-key infrastructure.
-Steps: persist tokens encrypted; never share across users; respect source-system permissions (never fetch what the user cannot access).</t>
+          <t>Purpose: support folder URLs / IDs that resolve to many documents, with an extension point for other DMS systems.
+Steps: implement base multi-doc connector; keep the SourceConnector interface as the only required surface for new connectors.</t>
         </is>
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>Encrypted token store</t>
+          <t>Generic multi-doc connector</t>
         </is>
       </c>
       <c r="F82" s="22" t="inlineStr">
@@ -7506,21 +7549,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G82" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G82" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>7.2,2.8</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="I82" s="17" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="J82" s="17" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="K82" s="17" t="n"/>
       <c r="L82" s="18" t="n">
@@ -7532,15 +7575,15 @@
         </is>
       </c>
       <c r="N82" s="19" t="n">
+        <v>46273</v>
+      </c>
+      <c r="O82" s="19" t="n">
         <v>46275</v>
-      </c>
-      <c r="O82" s="19" t="n">
-        <v>46276</v>
       </c>
       <c r="P82" s="3" t="n"/>
       <c r="Q82" s="3" t="inlineStr">
         <is>
-          <t>Tokens encrypted per user; no cross-user leak</t>
+          <t>New connector = implement interface only</t>
         </is>
       </c>
       <c r="R82" s="3" t="inlineStr"/>
@@ -7549,7 +7592,7 @@
     <row r="83" ht="75" customHeight="1">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>7.4</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -7559,18 +7602,18 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>Frontend: Add from SharePoint / Link flow</t>
+          <t>Encrypted per-user token storage</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Purpose: ship the operator UX for connect → folder pick → select → progress, then chat across the pulled set.
-Steps: add sources steps UI; show per-doc progress; ensure i18n for all locales; group pulled docs for chat/search.</t>
+          <t>Purpose: store connector OAuth tokens encrypted per user using existing encryption-key infrastructure.
+Steps: persist tokens encrypted; never share across users; respect source-system permissions (never fetch what the user cannot access).</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>Sources UI flow</t>
+          <t>Encrypted token store</t>
         </is>
       </c>
       <c r="F83" s="22" t="inlineStr">
@@ -7578,21 +7621,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G83" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G83" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H83" s="3" t="inlineStr">
         <is>
-          <t>7.2,7.3</t>
+          <t>7.2,2.8</t>
         </is>
       </c>
       <c r="I83" s="17" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="J83" s="17" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="K83" s="17" t="n"/>
       <c r="L83" s="18" t="n">
@@ -7600,32 +7643,28 @@
       </c>
       <c r="M83" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N83" s="19" t="n">
+        <v>46275</v>
+      </c>
+      <c r="O83" s="19" t="n">
         <v>46276</v>
-      </c>
-      <c r="O83" s="19" t="n">
-        <v>46281</v>
       </c>
       <c r="P83" s="3" t="n"/>
       <c r="Q83" s="3" t="inlineStr">
         <is>
-          <t>User can chat across the whole pulled set</t>
-        </is>
-      </c>
-      <c r="R83" s="3" t="inlineStr">
-        <is>
-          <t>i18n required for all locales</t>
-        </is>
-      </c>
+          <t>Tokens encrypted per user; no cross-user leak</t>
+        </is>
+      </c>
+      <c r="R83" s="3" t="inlineStr"/>
       <c r="S83" s="3" t="inlineStr"/>
     </row>
     <row r="84" ht="75" customHeight="1">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>7.6</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -7635,18 +7674,18 @@
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>docs/CONNECTORS.md + WP5 review</t>
+          <t>Frontend: Add from SharePoint / Link flow</t>
         </is>
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Purpose: document Entra scopes/consent and how to add a connector; close WP5 on acceptance criteria.
-Steps: write CONNECTORS.md; verify ACs; PR; human review stop.</t>
+          <t>Purpose: ship the operator UX for connect → folder pick → select → progress, then chat across the pulled set.
+Steps: add sources steps UI; show per-doc progress; ensure i18n for all locales; group pulled docs for chat/search.</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>docs/CONNECTORS.md; merged WP5</t>
+          <t>Sources UI flow</t>
         </is>
       </c>
       <c r="F84" s="22" t="inlineStr">
@@ -7661,14 +7700,14 @@
       </c>
       <c r="H84" s="3" t="inlineStr">
         <is>
-          <t>7.4,7.5</t>
+          <t>7.2,7.3</t>
         </is>
       </c>
       <c r="I84" s="17" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="J84" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K84" s="17" t="n"/>
       <c r="L84" s="18" t="n">
@@ -7676,49 +7715,53 @@
       </c>
       <c r="M84" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N84" s="19" t="n">
+        <v>46276</v>
+      </c>
+      <c r="O84" s="19" t="n">
         <v>46281</v>
-      </c>
-      <c r="O84" s="19" t="n">
-        <v>46282</v>
       </c>
       <c r="P84" s="3" t="n"/>
       <c r="Q84" s="3" t="inlineStr">
         <is>
-          <t>All WP5 acceptance criteria pass</t>
-        </is>
-      </c>
-      <c r="R84" s="3" t="inlineStr"/>
+          <t>User can chat across the whole pulled set</t>
+        </is>
+      </c>
+      <c r="R84" s="3" t="inlineStr">
+        <is>
+          <t>i18n required for all locales</t>
+        </is>
+      </c>
       <c r="S84" s="3" t="inlineStr"/>
     </row>
     <row r="85" ht="75" customHeight="1">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>7.6</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>WP6 — Doc Processing Benchmarks</t>
+          <t>WP5 — External Source Connectors</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>WP6 kickoff + enumerate supported types</t>
+          <t>docs/CONNECTORS.md + WP5 review</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Purpose: list what content-core actually supports today and what needs work (OCR, EPUB, upload HTML, etc.).
-Steps: inventory from real code/config; note gaps; create wp-6-benchmarks. Can run after WP0; needs target hardware for later measurement tasks.</t>
+          <t>Purpose: document Entra scopes/consent and how to add a connector; close WP5 on acceptance criteria.
+Steps: write CONNECTORS.md; verify ACs; PR; human review stop.</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Type inventory</t>
+          <t>docs/CONNECTORS.md; merged WP5</t>
         </is>
       </c>
       <c r="F85" s="22" t="inlineStr">
@@ -7726,14 +7769,14 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G85" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G85" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H85" s="3" t="inlineStr">
         <is>
-          <t>1.11</t>
+          <t>7.4,7.5</t>
         </is>
       </c>
       <c r="I85" s="17" t="n">
@@ -7752,28 +7795,24 @@
         </is>
       </c>
       <c r="N85" s="19" t="n">
-        <v>46266</v>
+        <v>46281</v>
       </c>
       <c r="O85" s="19" t="n">
-        <v>46267</v>
+        <v>46282</v>
       </c>
       <c r="P85" s="3" t="n"/>
       <c r="Q85" s="3" t="inlineStr">
         <is>
-          <t>Supported types documented from real code</t>
-        </is>
-      </c>
-      <c r="R85" s="3" t="inlineStr">
-        <is>
-          <t>No guessed client-facing numbers</t>
-        </is>
-      </c>
+          <t>All WP5 acceptance criteria pass</t>
+        </is>
+      </c>
+      <c r="R85" s="3" t="inlineStr"/>
       <c r="S85" s="3" t="inlineStr"/>
     </row>
     <row r="86" ht="75" customHeight="1">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -7783,18 +7822,18 @@
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>Build /benchmarks/ harness</t>
+          <t>WP6 kickoff + enumerate supported types</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>Purpose: produce repeatable measured metrics — not estimates — for ingestion, extraction, embedding, memory, and search/chat latency.
-Steps: build parameterized harness under /benchmarks/; output machine-readable reports.</t>
+          <t>Purpose: list what content-core actually supports today and what needs work (OCR, EPUB, upload HTML, etc.).
+Steps: inventory from real code/config; note gaps; create wp-6-benchmarks. Can run after WP0; needs target hardware for later measurement tasks.</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>/benchmarks/ harness</t>
+          <t>Type inventory</t>
         </is>
       </c>
       <c r="F86" s="22" t="inlineStr">
@@ -7802,21 +7841,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G86" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G86" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>1.11</t>
         </is>
       </c>
       <c r="I86" s="17" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="J86" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K86" s="17" t="n"/>
       <c r="L86" s="18" t="n">
@@ -7828,24 +7867,28 @@
         </is>
       </c>
       <c r="N86" s="19" t="n">
+        <v>46266</v>
+      </c>
+      <c r="O86" s="19" t="n">
         <v>46267</v>
-      </c>
-      <c r="O86" s="19" t="n">
-        <v>46270</v>
       </c>
       <c r="P86" s="3" t="n"/>
       <c r="Q86" s="3" t="inlineStr">
         <is>
-          <t>Harness runs repeatably and outputs a metrics report</t>
-        </is>
-      </c>
-      <c r="R86" s="3" t="inlineStr"/>
+          <t>Supported types documented from real code</t>
+        </is>
+      </c>
+      <c r="R86" s="3" t="inlineStr">
+        <is>
+          <t>No guessed client-facing numbers</t>
+        </is>
+      </c>
       <c r="S86" s="3" t="inlineStr"/>
     </row>
     <row r="87" ht="75" customHeight="1">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>8.2</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -7855,18 +7898,18 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>Assemble representative corpus</t>
+          <t>Build /benchmarks/ harness</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Purpose: find empirical slowdown/failure points across sizes and types.
-Steps: assemble small/medium/large/very-large docs plus scanned PDF, audio, and web page; ensure corpus licensing is clean for redistribution in-repo if needed.</t>
+          <t>Purpose: produce repeatable measured metrics — not estimates — for ingestion, extraction, embedding, memory, and search/chat latency.
+Steps: build parameterized harness under /benchmarks/; output machine-readable reports.</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>Fixed corpus under benchmarks/</t>
+          <t>/benchmarks/ harness</t>
         </is>
       </c>
       <c r="F87" s="22" t="inlineStr">
@@ -7881,14 +7924,14 @@
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="I87" s="17" t="n">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="J87" s="17" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="K87" s="17" t="n"/>
       <c r="L87" s="18" t="n">
@@ -7900,15 +7943,15 @@
         </is>
       </c>
       <c r="N87" s="19" t="n">
+        <v>46267</v>
+      </c>
+      <c r="O87" s="19" t="n">
         <v>46270</v>
-      </c>
-      <c r="O87" s="19" t="n">
-        <v>46273</v>
       </c>
       <c r="P87" s="3" t="n"/>
       <c r="Q87" s="3" t="inlineStr">
         <is>
-          <t>Corpus covers the size/type matrix</t>
+          <t>Harness runs repeatably and outputs a metrics report</t>
         </is>
       </c>
       <c r="R87" s="3" t="inlineStr"/>
@@ -7917,7 +7960,7 @@
     <row r="88" ht="75" customHeight="1">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>8.3</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
@@ -7927,18 +7970,18 @@
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>Define accuracy methodology</t>
+          <t>Assemble representative corpus</t>
         </is>
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>Purpose: define how accuracy is measured so client claims are defensible.
-Steps: specify extraction fidelity, retrieval relevance (labeled Q&amp;A), and chat groundedness methods; report per model tier.</t>
+          <t>Purpose: find empirical slowdown/failure points across sizes and types.
+Steps: assemble small/medium/large/very-large docs plus scanned PDF, audio, and web page; ensure corpus licensing is clean for redistribution in-repo if needed.</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>Accuracy method doc section</t>
+          <t>Fixed corpus under benchmarks/</t>
         </is>
       </c>
       <c r="F88" s="22" t="inlineStr">
@@ -7957,10 +8000,10 @@
         </is>
       </c>
       <c r="I88" s="17" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="J88" s="17" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="K88" s="17" t="n"/>
       <c r="L88" s="18" t="n">
@@ -7980,7 +8023,7 @@
       <c r="P88" s="3" t="n"/>
       <c r="Q88" s="3" t="inlineStr">
         <is>
-          <t>Accuracy reported as method + numbers</t>
+          <t>Corpus covers the size/type matrix</t>
         </is>
       </c>
       <c r="R88" s="3" t="inlineStr"/>
@@ -7989,7 +8032,7 @@
     <row r="89" ht="75" customHeight="1">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>8.3</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -7999,18 +8042,18 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>Run ≥2 hardware profiles</t>
+          <t>Define accuracy methodology</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Purpose: gather real numbers on bare-minimum and recommended hardware.
-Steps: run harness on both profiles; record figures; note local-model vs API-provider resource differences. Requires access to target hardware.</t>
+          <t>Purpose: define how accuracy is measured so client claims are defensible.
+Steps: specify extraction fidelity, retrieval relevance (labeled Q&amp;A), and chat groundedness methods; report per model tier.</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>Raw results JSON/CSV</t>
+          <t>Accuracy method doc section</t>
         </is>
       </c>
       <c r="F89" s="22" t="inlineStr">
@@ -8018,21 +8061,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G89" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G89" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H89" s="3" t="inlineStr">
         <is>
-          <t>8.2,8.3</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="I89" s="17" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="J89" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K89" s="17" t="n"/>
       <c r="L89" s="18" t="n">
@@ -8044,28 +8087,24 @@
         </is>
       </c>
       <c r="N89" s="19" t="n">
+        <v>46270</v>
+      </c>
+      <c r="O89" s="19" t="n">
         <v>46273</v>
-      </c>
-      <c r="O89" s="19" t="n">
-        <v>46276</v>
       </c>
       <c r="P89" s="3" t="n"/>
       <c r="Q89" s="3" t="inlineStr">
         <is>
-          <t>Real measured numbers for both profiles</t>
-        </is>
-      </c>
-      <c r="R89" s="3" t="inlineStr">
-        <is>
-          <t>Hardware access is a dependency</t>
-        </is>
-      </c>
+          <t>Accuracy reported as method + numbers</t>
+        </is>
+      </c>
+      <c r="R89" s="3" t="inlineStr"/>
       <c r="S89" s="3" t="inlineStr"/>
     </row>
     <row r="90" ht="75" customHeight="1">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
@@ -8075,18 +8114,18 @@
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>docs/PERFORMANCE_AND_SIZING.md + review</t>
+          <t>Run ≥2 hardware profiles</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Purpose: publish client-facing sizing guidance backed only by harness output.
-Steps: write types, limits, times, accuracy, min vs recommended hardware; peer review; merge.</t>
+          <t>Purpose: gather real numbers on bare-minimum and recommended hardware.
+Steps: run harness on both profiles; record figures; note local-model vs API-provider resource differences. Requires access to target hardware.</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>docs/PERFORMANCE_AND_SIZING.md</t>
+          <t>Raw results JSON/CSV</t>
         </is>
       </c>
       <c r="F90" s="22" t="inlineStr">
@@ -8094,21 +8133,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G90" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G90" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H90" s="3" t="inlineStr">
         <is>
-          <t>8.4</t>
+          <t>8.2,8.3</t>
         </is>
       </c>
       <c r="I90" s="17" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="J90" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K90" s="17" t="n"/>
       <c r="L90" s="18" t="n">
@@ -8120,45 +8159,49 @@
         </is>
       </c>
       <c r="N90" s="19" t="n">
+        <v>46273</v>
+      </c>
+      <c r="O90" s="19" t="n">
         <v>46276</v>
-      </c>
-      <c r="O90" s="19" t="n">
-        <v>46277</v>
       </c>
       <c r="P90" s="3" t="n"/>
       <c r="Q90" s="3" t="inlineStr">
         <is>
-          <t>Doc contains measured numbers only</t>
-        </is>
-      </c>
-      <c r="R90" s="3" t="inlineStr"/>
+          <t>Real measured numbers for both profiles</t>
+        </is>
+      </c>
+      <c r="R90" s="3" t="inlineStr">
+        <is>
+          <t>Hardware access is a dependency</t>
+        </is>
+      </c>
       <c r="S90" s="3" t="inlineStr"/>
     </row>
     <row r="91" ht="75" customHeight="1">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>WP7 — Cross-platform Packaging</t>
+          <t>WP6 — Doc Processing Benchmarks</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>WP7 kickoff</t>
+          <t>docs/PERFORMANCE_AND_SIZING.md + review</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Purpose: package the real authenticated + branded app, not the pre-WP2 password prototype.
-Steps: create wp-7-packaging only after WP2 and WP3 are on main.</t>
+          <t>Purpose: publish client-facing sizing guidance backed only by harness output.
+Steps: write types, limits, times, accuracy, min vs recommended hardware; peer review; merge.</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>Branch</t>
+          <t>docs/PERFORMANCE_AND_SIZING.md</t>
         </is>
       </c>
       <c r="F91" s="22" t="inlineStr">
@@ -8173,14 +8216,14 @@
       </c>
       <c r="H91" s="3" t="inlineStr">
         <is>
-          <t>5.6,4.10</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="I91" s="17" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J91" s="17" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="K91" s="17" t="n"/>
       <c r="L91" s="18" t="n">
@@ -8192,15 +8235,15 @@
         </is>
       </c>
       <c r="N91" s="19" t="n">
-        <v>46283</v>
+        <v>46276</v>
       </c>
       <c r="O91" s="19" t="n">
-        <v>46283</v>
+        <v>46277</v>
       </c>
       <c r="P91" s="3" t="n"/>
       <c r="Q91" s="3" t="inlineStr">
         <is>
-          <t>Starts only after branded + authenticated app exists</t>
+          <t>Doc contains measured numbers only</t>
         </is>
       </c>
       <c r="R91" s="3" t="inlineStr"/>
@@ -8209,7 +8252,7 @@
     <row r="92" ht="75" customHeight="1">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -8219,18 +8262,18 @@
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Verify Docker Compose on Windows + Linux</t>
+          <t>WP7 kickoff</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Purpose: make containers the recommended identical path on both OSes.
-Steps: verify docker-compose and Dockerfile.single on Docker Desktop/WSL2 and Linux; document as primary deploy path.</t>
+          <t>Purpose: package the real authenticated + branded app, not the pre-WP2 password prototype.
+Steps: create wp-7-packaging only after WP2 and WP3 are on main.</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>Verified container deploy</t>
+          <t>Branch</t>
         </is>
       </c>
       <c r="F92" s="22" t="inlineStr">
@@ -8238,21 +8281,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G92" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G92" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H92" s="3" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>5.6,4.10</t>
         </is>
       </c>
       <c r="I92" s="17" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="J92" s="17" t="n">
-        <v>2</v>
+        <v>0.25</v>
       </c>
       <c r="K92" s="17" t="n"/>
       <c r="L92" s="18" t="n">
@@ -8260,19 +8303,19 @@
       </c>
       <c r="M92" s="3" t="inlineStr">
         <is>
-          <t>DevOps / Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N92" s="19" t="n">
         <v>46283</v>
       </c>
       <c r="O92" s="19" t="n">
-        <v>46287</v>
+        <v>46283</v>
       </c>
       <c r="P92" s="3" t="n"/>
       <c r="Q92" s="3" t="inlineStr">
         <is>
-          <t>Container deployment verified on both OSes</t>
+          <t>Starts only after branded + authenticated app exists</t>
         </is>
       </c>
       <c r="R92" s="3" t="inlineStr"/>
@@ -8281,7 +8324,7 @@
     <row r="93" ht="75" customHeight="1">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>9.2</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -8291,18 +8334,18 @@
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>Native Linux install path (systemd)</t>
+          <t>Verify Docker Compose on Windows + Linux</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>Purpose: support customers who refuse containers.
-Steps: systemd units + install script; document dependencies for common distros; verify on at least one distro.</t>
+          <t>Purpose: make containers the recommended identical path on both OSes.
+Steps: verify docker-compose and Dockerfile.single on Docker Desktop/WSL2 and Linux; document as primary deploy path.</t>
         </is>
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>Linux native docs + scripts</t>
+          <t>Verified container deploy</t>
         </is>
       </c>
       <c r="F93" s="22" t="inlineStr">
@@ -8310,14 +8353,14 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G93" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G93" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H93" s="3" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="I93" s="17" t="n">
@@ -8336,15 +8379,15 @@
         </is>
       </c>
       <c r="N93" s="19" t="n">
+        <v>46283</v>
+      </c>
+      <c r="O93" s="19" t="n">
         <v>46287</v>
-      </c>
-      <c r="O93" s="19" t="n">
-        <v>46289</v>
       </c>
       <c r="P93" s="3" t="n"/>
       <c r="Q93" s="3" t="inlineStr">
         <is>
-          <t>Verified on ≥1 Linux distro</t>
+          <t>Container deployment verified on both OSes</t>
         </is>
       </c>
       <c r="R93" s="3" t="inlineStr"/>
@@ -8353,7 +8396,7 @@
     <row r="94" ht="75" customHeight="1">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>9.3</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -8363,18 +8406,18 @@
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>Native Windows Service path</t>
+          <t>Native Linux install path (systemd)</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Purpose: support Windows Server native installs.
-Steps: Windows Service wrapper; SurrealDB-on-Windows notes; frontend serve docs; verify on Windows Server or equivalent.</t>
+          <t>Purpose: support customers who refuse containers.
+Steps: systemd units + install script; document dependencies for common distros; verify on at least one distro.</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Windows native docs + scripts</t>
+          <t>Linux native docs + scripts</t>
         </is>
       </c>
       <c r="F94" s="22" t="inlineStr">
@@ -8416,7 +8459,7 @@
       <c r="P94" s="3" t="n"/>
       <c r="Q94" s="3" t="inlineStr">
         <is>
-          <t>Verified on Windows Server or equivalent</t>
+          <t>Verified on ≥1 Linux distro</t>
         </is>
       </c>
       <c r="R94" s="3" t="inlineStr"/>
@@ -8425,7 +8468,7 @@
     <row r="95" ht="75" customHeight="1">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>9.4</t>
+          <t>9.3</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -8435,18 +8478,18 @@
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>Installer helper CLI (interactive + non-interactive)</t>
+          <t>Native Windows Service path</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>Purpose: let a non-expert stand up a branded client instance without hand-editing half a dozen files.
-Steps: CLI for prereq check → collect brand/Entra/provider/DB/encryption → write config → migrate → start → health check; add scripted/non-interactive mode for repeatable installs.</t>
+          <t>Purpose: support Windows Server native installs.
+Steps: Windows Service wrapper; SurrealDB-on-Windows notes; frontend serve docs; verify on Windows Server or equivalent.</t>
         </is>
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>onboard/install CLI</t>
+          <t>Windows native docs + scripts</t>
         </is>
       </c>
       <c r="F95" s="22" t="inlineStr">
@@ -8454,21 +8497,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G95" s="20" t="inlineStr">
-        <is>
-          <t>Critical</t>
+      <c r="G95" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H95" s="3" t="inlineStr">
         <is>
-          <t>9.1,5.4</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="I95" s="17" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="J95" s="17" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K95" s="17" t="n"/>
       <c r="L95" s="18" t="n">
@@ -8476,32 +8519,28 @@
       </c>
       <c r="M95" s="3" t="inlineStr">
         <is>
-          <t>Backend Engineer</t>
+          <t>DevOps / Engineer</t>
         </is>
       </c>
       <c r="N95" s="19" t="n">
+        <v>46287</v>
+      </c>
+      <c r="O95" s="19" t="n">
         <v>46289</v>
-      </c>
-      <c r="O95" s="19" t="n">
-        <v>46295</v>
       </c>
       <c r="P95" s="3" t="n"/>
       <c r="Q95" s="3" t="inlineStr">
         <is>
-          <t>Full install in both modes; scripted branded client stand-up works</t>
-        </is>
-      </c>
-      <c r="R95" s="3" t="inlineStr">
-        <is>
-          <t>Deployment counterpart to WP3 theming</t>
-        </is>
-      </c>
+          <t>Verified on Windows Server or equivalent</t>
+        </is>
+      </c>
+      <c r="R95" s="3" t="inlineStr"/>
       <c r="S95" s="3" t="inlineStr"/>
     </row>
     <row r="96" ht="75" customHeight="1">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>9.5</t>
+          <t>9.4</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
@@ -8511,18 +8550,18 @@
       </c>
       <c r="C96" s="3" t="inlineStr">
         <is>
-          <t>docs/DEPLOYMENT.md + WP7 review</t>
+          <t>Installer helper CLI (interactive + non-interactive)</t>
         </is>
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>Purpose: one operator guide for container + native + CLI paths.
-Steps: write DEPLOYMENT.md; verify WP7 ACs; PR; human review.</t>
+          <t>Purpose: let a non-expert stand up a branded client instance without hand-editing half a dozen files.
+Steps: CLI for prereq check → collect brand/Entra/provider/DB/encryption → write config → migrate → start → health check; add scripted/non-interactive mode for repeatable installs.</t>
         </is>
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>docs/DEPLOYMENT.md</t>
+          <t>onboard/install CLI</t>
         </is>
       </c>
       <c r="F96" s="22" t="inlineStr">
@@ -8530,21 +8569,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G96" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G96" s="20" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
       <c r="H96" s="3" t="inlineStr">
         <is>
-          <t>9.2,9.3,9.4</t>
+          <t>9.1,5.4</t>
         </is>
       </c>
       <c r="I96" s="17" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="J96" s="17" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K96" s="17" t="n"/>
       <c r="L96" s="18" t="n">
@@ -8552,49 +8591,53 @@
       </c>
       <c r="M96" s="3" t="inlineStr">
         <is>
-          <t>Engineer</t>
+          <t>Backend Engineer</t>
         </is>
       </c>
       <c r="N96" s="19" t="n">
+        <v>46289</v>
+      </c>
+      <c r="O96" s="19" t="n">
         <v>46295</v>
-      </c>
-      <c r="O96" s="19" t="n">
-        <v>46296</v>
       </c>
       <c r="P96" s="3" t="n"/>
       <c r="Q96" s="3" t="inlineStr">
         <is>
-          <t>All WP7 acceptance criteria pass</t>
-        </is>
-      </c>
-      <c r="R96" s="3" t="inlineStr"/>
+          <t>Full install in both modes; scripted branded client stand-up works</t>
+        </is>
+      </c>
+      <c r="R96" s="3" t="inlineStr">
+        <is>
+          <t>Deployment counterpart to WP3 theming</t>
+        </is>
+      </c>
       <c r="S96" s="3" t="inlineStr"/>
     </row>
     <row r="97" ht="75" customHeight="1">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>9.5</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>WP8 — Onboarding &amp; In-app Help</t>
+          <t>WP7 — Cross-platform Packaging</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
-          <t>WP8 kickoff (LAST)</t>
+          <t>docs/DEPLOYMENT.md + WP7 review</t>
         </is>
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>Purpose: build onboarding against final flows only — wizard/tour copy must match the shipped product.
-Steps: create wp-8-onboarding after WP2/3/5/7 are stable on main.</t>
+          <t>Purpose: one operator guide for container + native + CLI paths.
+Steps: write DEPLOYMENT.md; verify WP7 ACs; PR; human review.</t>
         </is>
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>Branch</t>
+          <t>docs/DEPLOYMENT.md</t>
         </is>
       </c>
       <c r="F97" s="22" t="inlineStr">
@@ -8602,21 +8645,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G97" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G97" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H97" s="3" t="inlineStr">
         <is>
-          <t>9.5,7.6,5.6</t>
+          <t>9.2,9.3,9.4</t>
         </is>
       </c>
       <c r="I97" s="17" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J97" s="17" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="K97" s="17" t="n"/>
       <c r="L97" s="18" t="n">
@@ -8624,32 +8667,28 @@
       </c>
       <c r="M97" s="3" t="inlineStr">
         <is>
-          <t>Frontend Engineer</t>
+          <t>Engineer</t>
         </is>
       </c>
       <c r="N97" s="19" t="n">
-        <v>46297</v>
+        <v>46295</v>
       </c>
       <c r="O97" s="19" t="n">
-        <v>46297</v>
+        <v>46296</v>
       </c>
       <c r="P97" s="3" t="n"/>
       <c r="Q97" s="3" t="inlineStr">
         <is>
-          <t>Built against final UX</t>
-        </is>
-      </c>
-      <c r="R97" s="3" t="inlineStr">
-        <is>
-          <t>Must be last in the program sequence</t>
-        </is>
-      </c>
+          <t>All WP7 acceptance criteria pass</t>
+        </is>
+      </c>
+      <c r="R97" s="3" t="inlineStr"/>
       <c r="S97" s="3" t="inlineStr"/>
     </row>
     <row r="98" ht="75" customHeight="1">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
@@ -8659,18 +8698,18 @@
       </c>
       <c r="C98" s="3" t="inlineStr">
         <is>
-          <t>First-run / admin setup wizard</t>
+          <t>WP8 kickoff (LAST)</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>Purpose: take a fresh instance to a working configured app without tribal knowledge.
-Steps: detect fresh instance; guide providers/keys, models, brand (admin), connect a source, create first notebook; all copy via i18n.</t>
+          <t>Purpose: build onboarding against final flows only — wizard/tour copy must match the shipped product.
+Steps: create wp-8-onboarding after WP2/3/5/7 are stable on main.</t>
         </is>
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>Setup wizard</t>
+          <t>Branch</t>
         </is>
       </c>
       <c r="F98" s="22" t="inlineStr">
@@ -8678,21 +8717,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G98" s="16" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="G98" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="H98" s="3" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>9.5,7.6,5.6</t>
         </is>
       </c>
       <c r="I98" s="17" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="J98" s="17" t="n">
-        <v>3</v>
+        <v>0.25</v>
       </c>
       <c r="K98" s="17" t="n"/>
       <c r="L98" s="18" t="n">
@@ -8707,21 +8746,25 @@
         <v>46297</v>
       </c>
       <c r="O98" s="19" t="n">
-        <v>46302</v>
+        <v>46297</v>
       </c>
       <c r="P98" s="3" t="n"/>
       <c r="Q98" s="3" t="inlineStr">
         <is>
-          <t>Completing the wizard leaves a working configured app</t>
-        </is>
-      </c>
-      <c r="R98" s="3" t="inlineStr"/>
+          <t>Built against final UX</t>
+        </is>
+      </c>
+      <c r="R98" s="3" t="inlineStr">
+        <is>
+          <t>Must be last in the program sequence</t>
+        </is>
+      </c>
       <c r="S98" s="3" t="inlineStr"/>
     </row>
     <row r="99" ht="75" customHeight="1">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
@@ -8731,18 +8774,18 @@
       </c>
       <c r="C99" s="3" t="inlineStr">
         <is>
-          <t>User guided tour (core loop)</t>
+          <t>First-run / admin setup wizard</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>Purpose: teach the core loop — add source → search → chat → transform → podcast — with an accessible spotlight tour.
-Steps: implement dismissible/resumable tour; keep steps short; i18n all locales.</t>
+          <t>Purpose: take a fresh instance to a working configured app without tribal knowledge.
+Steps: detect fresh instance; guide providers/keys, models, brand (admin), connect a source, create first notebook; all copy via i18n.</t>
         </is>
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>Guided tour</t>
+          <t>Setup wizard</t>
         </is>
       </c>
       <c r="F99" s="22" t="inlineStr">
@@ -8757,14 +8800,14 @@
       </c>
       <c r="H99" s="3" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="I99" s="17" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="J99" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K99" s="17" t="n"/>
       <c r="L99" s="18" t="n">
@@ -8776,15 +8819,15 @@
         </is>
       </c>
       <c r="N99" s="19" t="n">
+        <v>46297</v>
+      </c>
+      <c r="O99" s="19" t="n">
         <v>46302</v>
-      </c>
-      <c r="O99" s="19" t="n">
-        <v>46304</v>
       </c>
       <c r="P99" s="3" t="n"/>
       <c r="Q99" s="3" t="inlineStr">
         <is>
-          <t>New user can complete the core-loop tour</t>
+          <t>Completing the wizard leaves a working configured app</t>
         </is>
       </c>
       <c r="R99" s="3" t="inlineStr"/>
@@ -8793,7 +8836,7 @@
     <row r="100" ht="75" customHeight="1">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
@@ -8803,18 +8846,18 @@
       </c>
       <c r="C100" s="3" t="inlineStr">
         <is>
-          <t>Contextual tooltips + empty states + help surface</t>
+          <t>User guided tour (core loop)</t>
         </is>
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>Purpose: remove dead-ends for new users on every main screen.
-Steps: tooltips on non-obvious controls; useful empty states; persistent help (docs, shortcuts, restart tour, BrandConfig support URL); all strings in i18n.</t>
+          <t>Purpose: teach the core loop — add source → search → chat → transform → podcast — with an accessible spotlight tour.
+Steps: implement dismissible/resumable tour; keep steps short; i18n all locales.</t>
         </is>
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>Tooltips/empty states/help</t>
+          <t>Guided tour</t>
         </is>
       </c>
       <c r="F100" s="22" t="inlineStr">
@@ -8822,21 +8865,21 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G100" s="21" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="G100" s="16" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="H100" s="3" t="inlineStr">
         <is>
-          <t>10.2</t>
+          <t>10.1</t>
         </is>
       </c>
       <c r="I100" s="17" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J100" s="17" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="K100" s="17" t="n"/>
       <c r="L100" s="18" t="n">
@@ -8848,28 +8891,24 @@
         </is>
       </c>
       <c r="N100" s="19" t="n">
+        <v>46302</v>
+      </c>
+      <c r="O100" s="19" t="n">
         <v>46304</v>
-      </c>
-      <c r="O100" s="19" t="n">
-        <v>46309</v>
       </c>
       <c r="P100" s="3" t="n"/>
       <c r="Q100" s="3" t="inlineStr">
         <is>
-          <t>All copy in i18n; help reachable everywhere</t>
-        </is>
-      </c>
-      <c r="R100" s="3" t="inlineStr">
-        <is>
-          <t>Locale parity required across all locales</t>
-        </is>
-      </c>
+          <t>New user can complete the core-loop tour</t>
+        </is>
+      </c>
+      <c r="R100" s="3" t="inlineStr"/>
       <c r="S100" s="3" t="inlineStr"/>
     </row>
     <row r="101" ht="75" customHeight="1">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>10.4</t>
+          <t>10.3</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -8879,18 +8918,18 @@
       </c>
       <c r="C101" s="3" t="inlineStr">
         <is>
-          <t>docs/ONBOARDING.md + program close review</t>
+          <t>Contextual tooltips + empty states + help surface</t>
         </is>
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>Purpose: document onboarding structure and verify program-level definition of done.
-Steps: write ONBOARDING.md; confirm a new client can be stood up by config + installer only (branded, Entra-auth’d, connectors, Windows/Linux) without per-client code rebuilds.</t>
+          <t>Purpose: remove dead-ends for new users on every main screen.
+Steps: tooltips on non-obvious controls; useful empty states; persistent help (docs, shortcuts, restart tour, BrandConfig support URL); all strings in i18n.</t>
         </is>
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>docs/ONBOARDING.md; program DoD check</t>
+          <t>Tooltips/empty states/help</t>
         </is>
       </c>
       <c r="F101" s="22" t="inlineStr">
@@ -8905,14 +8944,14 @@
       </c>
       <c r="H101" s="3" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>10.2</t>
         </is>
       </c>
       <c r="I101" s="17" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="J101" s="17" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="K101" s="17" t="n"/>
       <c r="L101" s="18" t="n">
@@ -8920,26 +8959,102 @@
       </c>
       <c r="M101" s="3" t="inlineStr">
         <is>
-          <t>Engineering Lead</t>
+          <t>Frontend Engineer</t>
         </is>
       </c>
       <c r="N101" s="19" t="n">
+        <v>46304</v>
+      </c>
+      <c r="O101" s="19" t="n">
         <v>46309</v>
-      </c>
-      <c r="O101" s="19" t="n">
-        <v>46310</v>
       </c>
       <c r="P101" s="3" t="n"/>
       <c r="Q101" s="3" t="inlineStr">
         <is>
+          <t>All copy in i18n; help reachable everywhere</t>
+        </is>
+      </c>
+      <c r="R101" s="3" t="inlineStr">
+        <is>
+          <t>Locale parity required across all locales</t>
+        </is>
+      </c>
+      <c r="S101" s="3" t="inlineStr"/>
+    </row>
+    <row r="102" ht="75" customHeight="1">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>10.4</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>WP8 — Onboarding &amp; In-app Help</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>docs/ONBOARDING.md + program close review</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>Purpose: document onboarding structure and verify program-level definition of done.
+Steps: write ONBOARDING.md; confirm a new client can be stood up by config + installer only (branded, Entra-auth’d, connectors, Windows/Linux) without per-client code rebuilds.</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>docs/ONBOARDING.md; program DoD check</t>
+        </is>
+      </c>
+      <c r="F102" s="22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="G102" s="21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H102" s="3" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="I102" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="J102" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K102" s="17" t="n"/>
+      <c r="L102" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M102" s="3" t="inlineStr">
+        <is>
+          <t>Engineering Lead</t>
+        </is>
+      </c>
+      <c r="N102" s="19" t="n">
+        <v>46309</v>
+      </c>
+      <c r="O102" s="19" t="n">
+        <v>46310</v>
+      </c>
+      <c r="P102" s="3" t="n"/>
+      <c r="Q102" s="3" t="inlineStr">
+        <is>
           <t>All WP8 ACs + program definition of done satisfied</t>
         </is>
       </c>
-      <c r="R101" s="3" t="inlineStr"/>
-      <c r="S101" s="3" t="inlineStr"/>
+      <c r="R102" s="3" t="inlineStr"/>
+      <c r="S102" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A5:S101"/>
+  <autoFilter ref="A5:S102"/>
   <mergeCells count="3">
     <mergeCell ref="A3:S3"/>
     <mergeCell ref="A2:S2"/>
@@ -9010,7 +9125,7 @@
           <t>Clean build reproducible from docs/DEV_SETUP.md</t>
         </is>
       </c>
-      <c r="C4" s="26" t="inlineStr">
+      <c r="C4" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9033,7 +9148,7 @@
           <t>upstream-base tag exists; upstream remote configured</t>
         </is>
       </c>
-      <c r="C5" s="26" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9060,7 +9175,7 @@
           <t>Characterization tests: ingestion, search, chat, notebook CRUD</t>
         </is>
       </c>
-      <c r="C6" s="26" t="inlineStr">
+      <c r="C6" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9083,7 +9198,7 @@
           <t>CI runs on PR and blocks merge on failure</t>
         </is>
       </c>
-      <c r="C7" s="26" t="inlineStr">
+      <c r="C7" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9106,7 +9221,7 @@
           <t>License scan runs in CI and passes</t>
         </is>
       </c>
-      <c r="C8" s="26" t="inlineStr">
+      <c r="C8" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9129,7 +9244,7 @@
           <t>LICENSE retains upstream copyright + our copyright</t>
         </is>
       </c>
-      <c r="C9" s="26" t="inlineStr">
+      <c r="C9" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9156,7 +9271,7 @@
           <t>THIRD-PARTY-NOTICES.md complete and reproducible</t>
         </is>
       </c>
-      <c r="C10" s="26" t="inlineStr">
+      <c r="C10" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9183,7 +9298,7 @@
           <t>SurrealDB BSL entry present and accurate</t>
         </is>
       </c>
-      <c r="C11" s="26" t="inlineStr">
+      <c r="C11" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9206,7 +9321,7 @@
           <t>pycountry unmodified; CI asserts</t>
         </is>
       </c>
-      <c r="C12" s="26" t="inlineStr">
+      <c r="C12" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9229,7 +9344,7 @@
           <t>docs/PROVIDER_TERMS.md exists</t>
         </is>
       </c>
-      <c r="C13" s="26" t="inlineStr">
+      <c r="C13" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9256,7 +9371,7 @@
           <t>No secrets committed; encryption key handling documented</t>
         </is>
       </c>
-      <c r="C14" s="26" t="inlineStr">
+      <c r="C14" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9279,7 +9394,7 @@
           <t>Tenancy model chosen and documented</t>
         </is>
       </c>
-      <c r="C15" s="26" t="inlineStr">
+      <c r="C15" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -9306,7 +9421,7 @@
           <t>Login via real Entra account E2E</t>
         </is>
       </c>
-      <c r="C16" s="27" t="inlineStr">
+      <c r="C16" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9329,7 +9444,7 @@
           <t>Every API request validates Entra JWT (iss/aud/sig/exp)</t>
         </is>
       </c>
-      <c r="C17" s="27" t="inlineStr">
+      <c r="C17" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9348,7 +9463,7 @@
           <t>Users JIT-provisioned; user record after first login</t>
         </is>
       </c>
-      <c r="C18" s="27" t="inlineStr">
+      <c r="C18" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9367,7 +9482,7 @@
           <t>Roles enforced on sensitive routes (403)</t>
         </is>
       </c>
-      <c r="C19" s="27" t="inlineStr">
+      <c r="C19" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9386,7 +9501,7 @@
           <t>Users only see own notebooks/sources</t>
         </is>
       </c>
-      <c r="C20" s="27" t="inlineStr">
+      <c r="C20" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9405,7 +9520,7 @@
           <t>Password provider still works as local-dev fallback</t>
         </is>
       </c>
-      <c r="C21" s="27" t="inlineStr">
+      <c r="C21" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9424,7 +9539,7 @@
           <t>Second provider needs no route-handler changes (stub)</t>
         </is>
       </c>
-      <c r="C22" s="27" t="inlineStr">
+      <c r="C22" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9443,7 +9558,7 @@
           <t>docs/AUTH.md complete</t>
         </is>
       </c>
-      <c r="C23" s="27" t="inlineStr">
+      <c r="C23" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9462,7 +9577,7 @@
           <t>FRONTEND_MAP.md complete with where-to-change table</t>
         </is>
       </c>
-      <c r="C24" s="27" t="inlineStr">
+      <c r="C24" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9481,7 +9596,7 @@
           <t>New client branded by config only (two brands, same build)</t>
         </is>
       </c>
-      <c r="C25" s="27" t="inlineStr">
+      <c r="C25" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9500,7 +9615,7 @@
           <t>Hardcoded brand strings/assets read from BrandConfig</t>
         </is>
       </c>
-      <c r="C26" s="27" t="inlineStr">
+      <c r="C26" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9519,7 +9634,7 @@
           <t>Dark/light both themed correctly</t>
         </is>
       </c>
-      <c r="C27" s="27" t="inlineStr">
+      <c r="C27" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9538,13 +9653,21 @@
           <t>Every router/endpoint documented with auth + models</t>
         </is>
       </c>
-      <c r="C28" s="27" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr"/>
-      <c r="E28" s="3" t="inlineStr"/>
+      <c r="C28" s="25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>docs/BACKEND_MAP.md</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>PR #55</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -9557,13 +9680,21 @@
           <t>Every domain model and graph documented</t>
         </is>
       </c>
-      <c r="C29" s="27" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
+      <c r="C29" s="25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>docs/BACKEND_MAP.md</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>PR #55</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -9576,13 +9707,21 @@
           <t>Five how-to-add-X playbooks present</t>
         </is>
       </c>
-      <c r="C30" s="27" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr"/>
-      <c r="E30" s="3" t="inlineStr"/>
+      <c r="C30" s="25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>docs/BACKEND_MAP.md</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>PR #55</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -9595,13 +9734,21 @@
           <t>New engineer can locate changes using only BACKEND_MAP</t>
         </is>
       </c>
-      <c r="C31" s="27" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
+      <c r="C31" s="25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>docs/BACKEND_MAP.md</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>tests/test_backend_map.py</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -9614,7 +9761,7 @@
           <t>SharePoint connect → folder → pull all supported docs</t>
         </is>
       </c>
-      <c r="C32" s="27" t="inlineStr">
+      <c r="C32" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9633,7 +9780,7 @@
           <t>Ingestion reuses existing pipeline</t>
         </is>
       </c>
-      <c r="C33" s="27" t="inlineStr">
+      <c r="C33" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9652,7 +9799,7 @@
           <t>Batch per-doc progress; single failure non-fatal</t>
         </is>
       </c>
-      <c r="C34" s="27" t="inlineStr">
+      <c r="C34" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9671,7 +9818,7 @@
           <t>Chat across whole pulled set</t>
         </is>
       </c>
-      <c r="C35" s="27" t="inlineStr">
+      <c r="C35" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9690,7 +9837,7 @@
           <t>Tokens encrypted per user; source permissions respected</t>
         </is>
       </c>
-      <c r="C36" s="27" t="inlineStr">
+      <c r="C36" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9709,7 +9856,7 @@
           <t>New connector = SourceConnector interface only</t>
         </is>
       </c>
-      <c r="C37" s="27" t="inlineStr">
+      <c r="C37" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9728,7 +9875,7 @@
           <t>docs/CONNECTORS.md complete</t>
         </is>
       </c>
-      <c r="C38" s="27" t="inlineStr">
+      <c r="C38" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9747,7 +9894,7 @@
           <t>Benchmark harness repeatable with metrics report</t>
         </is>
       </c>
-      <c r="C39" s="27" t="inlineStr">
+      <c r="C39" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9766,7 +9913,7 @@
           <t>PERFORMANCE_AND_SIZING.md has measured numbers (2 profiles)</t>
         </is>
       </c>
-      <c r="C40" s="27" t="inlineStr">
+      <c r="C40" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9785,7 +9932,7 @@
           <t>Supported types + tested size limits + failure points</t>
         </is>
       </c>
-      <c r="C41" s="27" t="inlineStr">
+      <c r="C41" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9804,7 +9951,7 @@
           <t>Accuracy methodology + results per model tier</t>
         </is>
       </c>
-      <c r="C42" s="27" t="inlineStr">
+      <c r="C42" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9823,7 +9970,7 @@
           <t>Min vs recommended hardware justified by numbers</t>
         </is>
       </c>
-      <c r="C43" s="27" t="inlineStr">
+      <c r="C43" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9842,7 +9989,7 @@
           <t>Container deploy verified Windows + Linux</t>
         </is>
       </c>
-      <c r="C44" s="27" t="inlineStr">
+      <c r="C44" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9861,7 +10008,7 @@
           <t>Native install documented/verified Linux + Windows</t>
         </is>
       </c>
-      <c r="C45" s="27" t="inlineStr">
+      <c r="C45" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9880,7 +10027,7 @@
           <t>Installer CLI full install interactive + non-interactive</t>
         </is>
       </c>
-      <c r="C46" s="27" t="inlineStr">
+      <c r="C46" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9899,7 +10046,7 @@
           <t>Scripted install stands up branded client E2E</t>
         </is>
       </c>
-      <c r="C47" s="27" t="inlineStr">
+      <c r="C47" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9918,7 +10065,7 @@
           <t>docs/DEPLOYMENT.md complete</t>
         </is>
       </c>
-      <c r="C48" s="27" t="inlineStr">
+      <c r="C48" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9937,7 +10084,7 @@
           <t>Fresh instance launches setup wizard → working app</t>
         </is>
       </c>
-      <c r="C49" s="27" t="inlineStr">
+      <c r="C49" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9956,7 +10103,7 @@
           <t>Guided tour of core loop completable</t>
         </is>
       </c>
-      <c r="C50" s="27" t="inlineStr">
+      <c r="C50" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9975,7 +10122,7 @@
           <t>Contextual tooltips; all copy in i18n</t>
         </is>
       </c>
-      <c r="C51" s="27" t="inlineStr">
+      <c r="C51" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -9994,7 +10141,7 @@
           <t>Every main screen useful empty state</t>
         </is>
       </c>
-      <c r="C52" s="27" t="inlineStr">
+      <c r="C52" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -10013,7 +10160,7 @@
           <t>Tour dismissible/resumable; help surface everywhere</t>
         </is>
       </c>
-      <c r="C53" s="27" t="inlineStr">
+      <c r="C53" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -10032,7 +10179,7 @@
           <t>docs/ONBOARDING.md complete</t>
         </is>
       </c>
-      <c r="C54" s="27" t="inlineStr">
+      <c r="C54" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -10051,7 +10198,7 @@
           <t>New client by config + installer only (no per-client rebuild)</t>
         </is>
       </c>
-      <c r="C55" s="27" t="inlineStr">
+      <c r="C55" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -10074,7 +10221,7 @@
           <t>Licensing compliant and drift-guarded</t>
         </is>
       </c>
-      <c r="C56" s="26" t="inlineStr">
+      <c r="C56" s="25" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
@@ -10097,7 +10244,7 @@
           <t>Real performance/sizing numbers for clients</t>
         </is>
       </c>
-      <c r="C57" s="27" t="inlineStr">
+      <c r="C57" s="26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -10120,17 +10267,21 @@
           <t>Backend + frontend fully mapped</t>
         </is>
       </c>
-      <c r="C58" s="27" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="C58" s="25" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>WP3a + WP4</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="inlineStr"/>
+          <t>docs/FRONTEND_MAP.md + docs/BACKEND_MAP.md</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>PR #55</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -10161,12 +10312,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="28" t="inlineStr">
+      <c r="A3" s="27" t="inlineStr">
         <is>
           <t>Topic</t>
         </is>
       </c>
-      <c r="B3" s="28" t="inlineStr">
+      <c r="B3" s="27" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>

</xml_diff>